<commit_message>
n4 yerine n5. BlokDairsel1Dondur-cd-v2
</commit_message>
<xml_diff>
--- a/KP-0-basic.xlsx
+++ b/KP-0-basic.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bingol/Documents/YU/YU-Projects/202304-BilisimDersleri/202401-YULearnt/hb-LightBoard/hb-Anlatim/KP-0-basic/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bingol/Documents/hb-git/git-IntroProgramming/AlgoritmikYaklasimlaProgramlamayaGiris/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F569287F-FCF7-2443-A2FF-00F0A87CC2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3024CB24-99EC-8849-9FD2-51E2B87CF694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" firstSheet="2" activeTab="7" xr2:uid="{43F04079-701F-514C-8FB9-C2E010C589CE}"/>
+    <workbookView xWindow="10880" yWindow="-21560" windowWidth="30240" windowHeight="18980" firstSheet="2" activeTab="6" xr2:uid="{43F04079-701F-514C-8FB9-C2E010C589CE}"/>
   </bookViews>
   <sheets>
     <sheet name="basliklar" sheetId="13" r:id="rId1"/>
@@ -2699,19 +2699,28 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2732,21 +2741,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2765,8 +2759,14 @@
     <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -8304,102 +8304,102 @@
     <row r="3" spans="1:45" s="74" customFormat="1" ht="19">
       <c r="A3" s="146"/>
       <c r="B3"/>
-      <c r="C3" s="209" t="s">
+      <c r="C3" s="208" t="s">
         <v>153</v>
       </c>
-      <c r="D3" s="209"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="209"/>
-      <c r="G3" s="209"/>
-      <c r="H3" s="209"/>
-      <c r="I3" s="209"/>
-      <c r="J3" s="209"/>
-      <c r="K3" s="209"/>
-      <c r="L3" s="209"/>
-      <c r="M3" s="209"/>
-      <c r="N3" s="209"/>
-      <c r="O3" s="209"/>
-      <c r="P3" s="209"/>
-      <c r="Q3" s="209"/>
-      <c r="R3" s="209"/>
-      <c r="S3" s="209"/>
-      <c r="T3" s="209"/>
+      <c r="D3" s="208"/>
+      <c r="E3" s="208"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="208"/>
+      <c r="H3" s="208"/>
+      <c r="I3" s="208"/>
+      <c r="J3" s="208"/>
+      <c r="K3" s="208"/>
+      <c r="L3" s="208"/>
+      <c r="M3" s="208"/>
+      <c r="N3" s="208"/>
+      <c r="O3" s="208"/>
+      <c r="P3" s="208"/>
+      <c r="Q3" s="208"/>
+      <c r="R3" s="208"/>
+      <c r="S3" s="208"/>
+      <c r="T3" s="208"/>
       <c r="U3" s="146"/>
       <c r="V3"/>
-      <c r="W3" s="209" t="s">
+      <c r="W3" s="208" t="s">
         <v>154</v>
       </c>
-      <c r="X3" s="209"/>
-      <c r="Y3" s="209"/>
-      <c r="Z3" s="209"/>
-      <c r="AA3" s="209"/>
-      <c r="AB3" s="209"/>
-      <c r="AC3" s="209"/>
-      <c r="AD3" s="209"/>
-      <c r="AE3" s="209"/>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="209"/>
-      <c r="AH3" s="209"/>
-      <c r="AI3" s="209"/>
-      <c r="AJ3" s="209"/>
-      <c r="AK3" s="209"/>
-      <c r="AL3" s="209"/>
-      <c r="AM3" s="209"/>
-      <c r="AN3" s="209"/>
-      <c r="AO3" s="209"/>
-      <c r="AP3" s="209"/>
-      <c r="AQ3" s="209"/>
+      <c r="X3" s="208"/>
+      <c r="Y3" s="208"/>
+      <c r="Z3" s="208"/>
+      <c r="AA3" s="208"/>
+      <c r="AB3" s="208"/>
+      <c r="AC3" s="208"/>
+      <c r="AD3" s="208"/>
+      <c r="AE3" s="208"/>
+      <c r="AF3" s="208"/>
+      <c r="AG3" s="208"/>
+      <c r="AH3" s="208"/>
+      <c r="AI3" s="208"/>
+      <c r="AJ3" s="208"/>
+      <c r="AK3" s="208"/>
+      <c r="AL3" s="208"/>
+      <c r="AM3" s="208"/>
+      <c r="AN3" s="208"/>
+      <c r="AO3" s="208"/>
+      <c r="AP3" s="208"/>
+      <c r="AQ3" s="208"/>
       <c r="AR3" s="146"/>
       <c r="AS3"/>
     </row>
     <row r="4" spans="1:45" s="74" customFormat="1" ht="19">
       <c r="A4" s="146"/>
       <c r="B4"/>
-      <c r="C4" s="209" t="s">
+      <c r="C4" s="208" t="s">
         <v>155</v>
       </c>
-      <c r="D4" s="209"/>
-      <c r="E4" s="209"/>
-      <c r="F4" s="209"/>
-      <c r="G4" s="209"/>
-      <c r="H4" s="209"/>
-      <c r="I4" s="209"/>
-      <c r="J4" s="209"/>
-      <c r="K4" s="209"/>
-      <c r="L4" s="209"/>
-      <c r="M4" s="209"/>
-      <c r="N4" s="209"/>
-      <c r="O4" s="209"/>
-      <c r="P4" s="209"/>
-      <c r="Q4" s="209"/>
-      <c r="R4" s="209"/>
-      <c r="S4" s="209"/>
-      <c r="T4" s="209"/>
+      <c r="D4" s="208"/>
+      <c r="E4" s="208"/>
+      <c r="F4" s="208"/>
+      <c r="G4" s="208"/>
+      <c r="H4" s="208"/>
+      <c r="I4" s="208"/>
+      <c r="J4" s="208"/>
+      <c r="K4" s="208"/>
+      <c r="L4" s="208"/>
+      <c r="M4" s="208"/>
+      <c r="N4" s="208"/>
+      <c r="O4" s="208"/>
+      <c r="P4" s="208"/>
+      <c r="Q4" s="208"/>
+      <c r="R4" s="208"/>
+      <c r="S4" s="208"/>
+      <c r="T4" s="208"/>
       <c r="U4" s="146"/>
       <c r="V4"/>
-      <c r="W4" s="217" t="s">
+      <c r="W4" s="210" t="s">
         <v>201</v>
       </c>
-      <c r="X4" s="217"/>
-      <c r="Y4" s="217"/>
-      <c r="Z4" s="217"/>
-      <c r="AA4" s="217"/>
-      <c r="AB4" s="217"/>
-      <c r="AC4" s="217"/>
-      <c r="AD4" s="217"/>
-      <c r="AE4" s="217"/>
-      <c r="AF4" s="217"/>
-      <c r="AG4" s="217"/>
-      <c r="AH4" s="217"/>
-      <c r="AI4" s="217"/>
-      <c r="AJ4" s="217"/>
-      <c r="AK4" s="217"/>
-      <c r="AL4" s="217"/>
-      <c r="AM4" s="217"/>
-      <c r="AN4" s="217"/>
-      <c r="AO4" s="217"/>
-      <c r="AP4" s="217"/>
-      <c r="AQ4" s="217"/>
+      <c r="X4" s="210"/>
+      <c r="Y4" s="210"/>
+      <c r="Z4" s="210"/>
+      <c r="AA4" s="210"/>
+      <c r="AB4" s="210"/>
+      <c r="AC4" s="210"/>
+      <c r="AD4" s="210"/>
+      <c r="AE4" s="210"/>
+      <c r="AF4" s="210"/>
+      <c r="AG4" s="210"/>
+      <c r="AH4" s="210"/>
+      <c r="AI4" s="210"/>
+      <c r="AJ4" s="210"/>
+      <c r="AK4" s="210"/>
+      <c r="AL4" s="210"/>
+      <c r="AM4" s="210"/>
+      <c r="AN4" s="210"/>
+      <c r="AO4" s="210"/>
+      <c r="AP4" s="210"/>
+      <c r="AQ4" s="210"/>
       <c r="AR4" s="146"/>
       <c r="AS4"/>
     </row>
@@ -8656,18 +8656,18 @@
       <c r="G10" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="210" t="s">
+      <c r="I10" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="J10" s="210"/>
-      <c r="K10" s="210"/>
-      <c r="L10" s="210"/>
-      <c r="M10" s="210"/>
-      <c r="N10" s="210"/>
-      <c r="O10" s="210"/>
-      <c r="P10" s="210"/>
-      <c r="Q10" s="210"/>
-      <c r="R10" s="210"/>
+      <c r="J10" s="209"/>
+      <c r="K10" s="209"/>
+      <c r="L10" s="209"/>
+      <c r="M10" s="209"/>
+      <c r="N10" s="209"/>
+      <c r="O10" s="209"/>
+      <c r="P10" s="209"/>
+      <c r="Q10" s="209"/>
+      <c r="R10" s="209"/>
       <c r="T10" s="53" t="s">
         <v>17</v>
       </c>
@@ -8677,10 +8677,10 @@
       </c>
       <c r="X10" s="4"/>
       <c r="Y10" s="32"/>
-      <c r="Z10" s="211" t="s">
+      <c r="Z10" s="214" t="s">
         <v>156</v>
       </c>
-      <c r="AA10" s="211"/>
+      <c r="AA10" s="214"/>
       <c r="AB10" s="32"/>
       <c r="AC10" s="98" t="s">
         <v>14</v>
@@ -8688,18 +8688,18 @@
       <c r="AD10" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="AF10" s="210" t="s">
+      <c r="AF10" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="AG10" s="210"/>
-      <c r="AH10" s="210"/>
-      <c r="AI10" s="210"/>
-      <c r="AJ10" s="210"/>
-      <c r="AK10" s="210"/>
-      <c r="AL10" s="210"/>
-      <c r="AM10" s="210"/>
-      <c r="AN10" s="210"/>
-      <c r="AO10" s="210"/>
+      <c r="AG10" s="209"/>
+      <c r="AH10" s="209"/>
+      <c r="AI10" s="209"/>
+      <c r="AJ10" s="209"/>
+      <c r="AK10" s="209"/>
+      <c r="AL10" s="209"/>
+      <c r="AM10" s="209"/>
+      <c r="AN10" s="209"/>
+      <c r="AO10" s="209"/>
       <c r="AP10" s="32"/>
       <c r="AQ10" s="53" t="s">
         <v>17</v>
@@ -11812,38 +11812,38 @@
     </row>
     <row r="3" spans="1:32" s="73" customFormat="1" ht="18">
       <c r="A3" s="146"/>
-      <c r="C3" s="217" t="s">
+      <c r="C3" s="210" t="s">
         <v>286</v>
       </c>
-      <c r="D3" s="217"/>
-      <c r="E3" s="217"/>
-      <c r="F3" s="217"/>
-      <c r="G3" s="217"/>
-      <c r="H3" s="217"/>
+      <c r="D3" s="210"/>
+      <c r="E3" s="210"/>
+      <c r="F3" s="210"/>
+      <c r="G3" s="210"/>
+      <c r="H3" s="210"/>
       <c r="I3" s="146"/>
-      <c r="K3" s="217" t="s">
+      <c r="K3" s="210" t="s">
         <v>286</v>
       </c>
-      <c r="L3" s="217"/>
-      <c r="M3" s="217"/>
-      <c r="N3" s="217"/>
-      <c r="O3" s="217"/>
-      <c r="P3" s="217"/>
-      <c r="Q3" s="217"/>
-      <c r="R3" s="217"/>
-      <c r="S3" s="217"/>
+      <c r="L3" s="210"/>
+      <c r="M3" s="210"/>
+      <c r="N3" s="210"/>
+      <c r="O3" s="210"/>
+      <c r="P3" s="210"/>
+      <c r="Q3" s="210"/>
+      <c r="R3" s="210"/>
+      <c r="S3" s="210"/>
       <c r="T3" s="146"/>
-      <c r="V3" s="217" t="s">
+      <c r="V3" s="210" t="s">
         <v>286</v>
       </c>
-      <c r="W3" s="217"/>
-      <c r="X3" s="217"/>
-      <c r="Y3" s="217"/>
-      <c r="Z3" s="217"/>
-      <c r="AA3" s="217"/>
-      <c r="AB3" s="217"/>
-      <c r="AC3" s="217"/>
-      <c r="AD3" s="217"/>
+      <c r="W3" s="210"/>
+      <c r="X3" s="210"/>
+      <c r="Y3" s="210"/>
+      <c r="Z3" s="210"/>
+      <c r="AA3" s="210"/>
+      <c r="AB3" s="210"/>
+      <c r="AC3" s="210"/>
+      <c r="AD3" s="210"/>
       <c r="AE3" s="146"/>
     </row>
     <row r="4" spans="1:32" s="73" customFormat="1" ht="18">
@@ -11870,40 +11870,40 @@
     <row r="5" spans="1:32" ht="19">
       <c r="A5" s="146"/>
       <c r="B5" s="74"/>
-      <c r="C5" s="217" t="s">
+      <c r="C5" s="210" t="s">
         <v>285</v>
       </c>
-      <c r="D5" s="217"/>
-      <c r="E5" s="217"/>
-      <c r="F5" s="217"/>
-      <c r="G5" s="217"/>
-      <c r="H5" s="217"/>
+      <c r="D5" s="210"/>
+      <c r="E5" s="210"/>
+      <c r="F5" s="210"/>
+      <c r="G5" s="210"/>
+      <c r="H5" s="210"/>
       <c r="I5" s="146"/>
       <c r="J5" s="74"/>
-      <c r="K5" s="217" t="s">
+      <c r="K5" s="210" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="217"/>
-      <c r="M5" s="217"/>
-      <c r="N5" s="217"/>
-      <c r="O5" s="217"/>
-      <c r="P5" s="217"/>
-      <c r="Q5" s="217"/>
-      <c r="R5" s="217"/>
-      <c r="S5" s="217"/>
+      <c r="L5" s="210"/>
+      <c r="M5" s="210"/>
+      <c r="N5" s="210"/>
+      <c r="O5" s="210"/>
+      <c r="P5" s="210"/>
+      <c r="Q5" s="210"/>
+      <c r="R5" s="210"/>
+      <c r="S5" s="210"/>
       <c r="T5" s="146"/>
       <c r="U5" s="74"/>
-      <c r="V5" s="217" t="s">
+      <c r="V5" s="210" t="s">
         <v>287</v>
       </c>
-      <c r="W5" s="217"/>
-      <c r="X5" s="217"/>
-      <c r="Y5" s="217"/>
-      <c r="Z5" s="217"/>
-      <c r="AA5" s="217"/>
-      <c r="AB5" s="217"/>
-      <c r="AC5" s="217"/>
-      <c r="AD5" s="217"/>
+      <c r="W5" s="210"/>
+      <c r="X5" s="210"/>
+      <c r="Y5" s="210"/>
+      <c r="Z5" s="210"/>
+      <c r="AA5" s="210"/>
+      <c r="AB5" s="210"/>
+      <c r="AC5" s="210"/>
+      <c r="AD5" s="210"/>
       <c r="AE5" s="146"/>
       <c r="AF5" s="74"/>
     </row>
@@ -11926,11 +11926,11 @@
       <c r="E7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="218" t="s">
+      <c r="F7" s="211" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="219"/>
-      <c r="H7" s="220"/>
+      <c r="G7" s="212"/>
+      <c r="H7" s="213"/>
       <c r="I7" s="146"/>
       <c r="K7" s="161" t="s">
         <v>14</v>
@@ -11938,12 +11938,12 @@
       <c r="L7" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="N7" s="211" t="s">
+      <c r="N7" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="211"/>
-      <c r="P7" s="211"/>
-      <c r="Q7" s="211"/>
+      <c r="O7" s="214"/>
+      <c r="P7" s="214"/>
+      <c r="Q7" s="214"/>
       <c r="S7" s="4" t="s">
         <v>17</v>
       </c>
@@ -11954,12 +11954,12 @@
       <c r="W7" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="Y7" s="218" t="s">
+      <c r="Y7" s="211" t="s">
         <v>16</v>
       </c>
-      <c r="Z7" s="219"/>
-      <c r="AA7" s="219"/>
-      <c r="AB7" s="220"/>
+      <c r="Z7" s="212"/>
+      <c r="AA7" s="212"/>
+      <c r="AB7" s="213"/>
       <c r="AD7" s="4" t="s">
         <v>17</v>
       </c>
@@ -12472,27 +12472,27 @@
       <c r="K21" s="161" t="s">
         <v>14</v>
       </c>
-      <c r="L21" s="221" t="s">
+      <c r="L21" s="206" t="s">
         <v>248</v>
       </c>
-      <c r="M21" s="221"/>
-      <c r="N21" s="221"/>
-      <c r="O21" s="221"/>
-      <c r="P21" s="221"/>
-      <c r="Q21" s="221"/>
-      <c r="R21" s="221"/>
-      <c r="S21" s="221"/>
+      <c r="M21" s="206"/>
+      <c r="N21" s="206"/>
+      <c r="O21" s="206"/>
+      <c r="P21" s="206"/>
+      <c r="Q21" s="206"/>
+      <c r="R21" s="206"/>
+      <c r="S21" s="206"/>
       <c r="T21" s="146"/>
-      <c r="W21" s="221" t="s">
+      <c r="W21" s="206" t="s">
         <v>265</v>
       </c>
-      <c r="X21" s="221"/>
-      <c r="Y21" s="221"/>
-      <c r="Z21" s="221"/>
-      <c r="AA21" s="221"/>
-      <c r="AB21" s="221"/>
-      <c r="AC21" s="221"/>
-      <c r="AD21" s="221"/>
+      <c r="X21" s="206"/>
+      <c r="Y21" s="206"/>
+      <c r="Z21" s="206"/>
+      <c r="AA21" s="206"/>
+      <c r="AB21" s="206"/>
+      <c r="AC21" s="206"/>
+      <c r="AD21" s="206"/>
       <c r="AE21" s="146"/>
     </row>
     <row r="22" spans="1:32">
@@ -12501,60 +12501,60 @@
       <c r="K22" s="163">
         <v>1</v>
       </c>
-      <c r="L22" s="214" t="s">
+      <c r="L22" s="217" t="s">
         <v>288</v>
       </c>
-      <c r="M22" s="215"/>
-      <c r="N22" s="215"/>
-      <c r="O22" s="215"/>
-      <c r="P22" s="215"/>
-      <c r="Q22" s="215"/>
-      <c r="R22" s="215"/>
-      <c r="S22" s="215"/>
+      <c r="M22" s="218"/>
+      <c r="N22" s="218"/>
+      <c r="O22" s="218"/>
+      <c r="P22" s="218"/>
+      <c r="Q22" s="218"/>
+      <c r="R22" s="218"/>
+      <c r="S22" s="218"/>
       <c r="T22" s="146"/>
       <c r="V22" s="123">
         <v>1</v>
       </c>
-      <c r="W22" s="216" t="s">
+      <c r="W22" s="219" t="s">
         <v>166</v>
       </c>
-      <c r="X22" s="216"/>
-      <c r="Y22" s="216"/>
-      <c r="Z22" s="216"/>
-      <c r="AA22" s="216"/>
-      <c r="AB22" s="216"/>
-      <c r="AC22" s="216"/>
-      <c r="AD22" s="216"/>
+      <c r="X22" s="219"/>
+      <c r="Y22" s="219"/>
+      <c r="Z22" s="219"/>
+      <c r="AA22" s="219"/>
+      <c r="AB22" s="219"/>
+      <c r="AC22" s="219"/>
+      <c r="AD22" s="219"/>
       <c r="AE22" s="146"/>
     </row>
     <row r="23" spans="1:32">
       <c r="A23" s="146"/>
       <c r="I23" s="146"/>
       <c r="K23" s="162"/>
-      <c r="L23" s="212" t="s">
+      <c r="L23" s="215" t="s">
         <v>289</v>
       </c>
-      <c r="M23" s="212"/>
-      <c r="N23" s="212"/>
-      <c r="O23" s="212"/>
-      <c r="P23" s="212"/>
-      <c r="Q23" s="212"/>
-      <c r="R23" s="212"/>
-      <c r="S23" s="212"/>
+      <c r="M23" s="215"/>
+      <c r="N23" s="215"/>
+      <c r="O23" s="215"/>
+      <c r="P23" s="215"/>
+      <c r="Q23" s="215"/>
+      <c r="R23" s="215"/>
+      <c r="S23" s="215"/>
       <c r="T23" s="146"/>
       <c r="V23" s="123">
         <v>2</v>
       </c>
-      <c r="W23" s="216" t="s">
+      <c r="W23" s="219" t="s">
         <v>167</v>
       </c>
-      <c r="X23" s="216"/>
-      <c r="Y23" s="216"/>
-      <c r="Z23" s="216"/>
-      <c r="AA23" s="216"/>
-      <c r="AB23" s="216"/>
-      <c r="AC23" s="216"/>
-      <c r="AD23" s="216"/>
+      <c r="X23" s="219"/>
+      <c r="Y23" s="219"/>
+      <c r="Z23" s="219"/>
+      <c r="AA23" s="219"/>
+      <c r="AB23" s="219"/>
+      <c r="AC23" s="219"/>
+      <c r="AD23" s="219"/>
       <c r="AE23" s="146"/>
     </row>
     <row r="24" spans="1:32">
@@ -12563,16 +12563,16 @@
       <c r="K24" s="123">
         <v>2</v>
       </c>
-      <c r="L24" s="213" t="s">
+      <c r="L24" s="216" t="s">
         <v>290</v>
       </c>
-      <c r="M24" s="213"/>
-      <c r="N24" s="213"/>
-      <c r="O24" s="213"/>
-      <c r="P24" s="213"/>
-      <c r="Q24" s="213"/>
-      <c r="R24" s="213"/>
-      <c r="S24" s="213"/>
+      <c r="M24" s="216"/>
+      <c r="N24" s="216"/>
+      <c r="O24" s="216"/>
+      <c r="P24" s="216"/>
+      <c r="Q24" s="216"/>
+      <c r="R24" s="216"/>
+      <c r="S24" s="216"/>
       <c r="T24" s="146"/>
       <c r="Y24" s="1"/>
       <c r="Z24" s="19"/>
@@ -12586,16 +12586,16 @@
       <c r="K25" s="123">
         <v>3</v>
       </c>
-      <c r="L25" s="213" t="s">
+      <c r="L25" s="216" t="s">
         <v>291</v>
       </c>
-      <c r="M25" s="213"/>
-      <c r="N25" s="213"/>
-      <c r="O25" s="213"/>
-      <c r="P25" s="213"/>
-      <c r="Q25" s="213"/>
-      <c r="R25" s="213"/>
-      <c r="S25" s="213"/>
+      <c r="M25" s="216"/>
+      <c r="N25" s="216"/>
+      <c r="O25" s="216"/>
+      <c r="P25" s="216"/>
+      <c r="Q25" s="216"/>
+      <c r="R25" s="216"/>
+      <c r="S25" s="216"/>
       <c r="T25" s="146"/>
       <c r="W25" s="77" t="s">
         <v>24</v>
@@ -13219,6 +13219,12 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="L23:S23"/>
+    <mergeCell ref="L24:S24"/>
+    <mergeCell ref="L25:S25"/>
+    <mergeCell ref="L22:S22"/>
+    <mergeCell ref="W22:AD22"/>
+    <mergeCell ref="W23:AD23"/>
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="Y7:AB7"/>
     <mergeCell ref="F7:H7"/>
@@ -13230,12 +13236,6 @@
     <mergeCell ref="K5:S5"/>
     <mergeCell ref="N7:Q7"/>
     <mergeCell ref="W21:AD21"/>
-    <mergeCell ref="L23:S23"/>
-    <mergeCell ref="L24:S24"/>
-    <mergeCell ref="L25:S25"/>
-    <mergeCell ref="L22:S22"/>
-    <mergeCell ref="W22:AD22"/>
-    <mergeCell ref="W23:AD23"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="W26" r:id="rId1" xr:uid="{4F5EB8FC-141A-4D4E-BEF7-FFB87DF5DFDC}"/>
@@ -13336,49 +13336,49 @@
     <row r="3" spans="1:41" s="74" customFormat="1" ht="19">
       <c r="A3" s="146"/>
       <c r="B3"/>
-      <c r="C3" s="209" t="s">
+      <c r="C3" s="208" t="s">
         <v>252</v>
       </c>
-      <c r="D3" s="209"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="209"/>
-      <c r="G3" s="209"/>
-      <c r="H3" s="209"/>
-      <c r="I3" s="209"/>
-      <c r="J3" s="209"/>
-      <c r="K3" s="209"/>
-      <c r="L3" s="209"/>
-      <c r="M3" s="209"/>
+      <c r="D3" s="208"/>
+      <c r="E3" s="208"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="208"/>
+      <c r="H3" s="208"/>
+      <c r="I3" s="208"/>
+      <c r="J3" s="208"/>
+      <c r="K3" s="208"/>
+      <c r="L3" s="208"/>
+      <c r="M3" s="208"/>
       <c r="N3" s="146"/>
       <c r="O3"/>
-      <c r="P3" s="209" t="s">
+      <c r="P3" s="208" t="s">
         <v>252</v>
       </c>
-      <c r="Q3" s="209"/>
-      <c r="R3" s="209"/>
-      <c r="S3" s="209"/>
-      <c r="T3" s="209"/>
-      <c r="U3" s="209"/>
-      <c r="V3" s="209"/>
-      <c r="W3" s="209"/>
-      <c r="X3" s="209"/>
-      <c r="Y3" s="209"/>
-      <c r="Z3" s="209"/>
+      <c r="Q3" s="208"/>
+      <c r="R3" s="208"/>
+      <c r="S3" s="208"/>
+      <c r="T3" s="208"/>
+      <c r="U3" s="208"/>
+      <c r="V3" s="208"/>
+      <c r="W3" s="208"/>
+      <c r="X3" s="208"/>
+      <c r="Y3" s="208"/>
+      <c r="Z3" s="208"/>
       <c r="AA3" s="146"/>
       <c r="AB3"/>
-      <c r="AC3" s="209" t="s">
+      <c r="AC3" s="208" t="s">
         <v>252</v>
       </c>
-      <c r="AD3" s="209"/>
-      <c r="AE3" s="209"/>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="209"/>
-      <c r="AH3" s="209"/>
-      <c r="AI3" s="209"/>
-      <c r="AJ3" s="209"/>
-      <c r="AK3" s="209"/>
-      <c r="AL3" s="209"/>
-      <c r="AM3" s="209"/>
+      <c r="AD3" s="208"/>
+      <c r="AE3" s="208"/>
+      <c r="AF3" s="208"/>
+      <c r="AG3" s="208"/>
+      <c r="AH3" s="208"/>
+      <c r="AI3" s="208"/>
+      <c r="AJ3" s="208"/>
+      <c r="AK3" s="208"/>
+      <c r="AL3" s="208"/>
+      <c r="AM3" s="208"/>
       <c r="AN3" s="146"/>
       <c r="AO3"/>
     </row>
@@ -13428,49 +13428,49 @@
     <row r="5" spans="1:41" s="74" customFormat="1" ht="19">
       <c r="A5" s="146"/>
       <c r="B5"/>
-      <c r="C5" s="209" t="s">
+      <c r="C5" s="208" t="s">
         <v>253</v>
       </c>
-      <c r="D5" s="209"/>
-      <c r="E5" s="209"/>
-      <c r="F5" s="209"/>
-      <c r="G5" s="209"/>
-      <c r="H5" s="209"/>
-      <c r="I5" s="209"/>
-      <c r="J5" s="209"/>
-      <c r="K5" s="209"/>
-      <c r="L5" s="209"/>
-      <c r="M5" s="209"/>
+      <c r="D5" s="208"/>
+      <c r="E5" s="208"/>
+      <c r="F5" s="208"/>
+      <c r="G5" s="208"/>
+      <c r="H5" s="208"/>
+      <c r="I5" s="208"/>
+      <c r="J5" s="208"/>
+      <c r="K5" s="208"/>
+      <c r="L5" s="208"/>
+      <c r="M5" s="208"/>
       <c r="N5" s="146"/>
       <c r="O5"/>
-      <c r="P5" s="209" t="s">
+      <c r="P5" s="208" t="s">
         <v>254</v>
       </c>
-      <c r="Q5" s="209"/>
-      <c r="R5" s="209"/>
-      <c r="S5" s="209"/>
-      <c r="T5" s="209"/>
-      <c r="U5" s="209"/>
-      <c r="V5" s="209"/>
-      <c r="W5" s="209"/>
-      <c r="X5" s="209"/>
-      <c r="Y5" s="209"/>
-      <c r="Z5" s="209"/>
+      <c r="Q5" s="208"/>
+      <c r="R5" s="208"/>
+      <c r="S5" s="208"/>
+      <c r="T5" s="208"/>
+      <c r="U5" s="208"/>
+      <c r="V5" s="208"/>
+      <c r="W5" s="208"/>
+      <c r="X5" s="208"/>
+      <c r="Y5" s="208"/>
+      <c r="Z5" s="208"/>
       <c r="AA5" s="146"/>
       <c r="AB5"/>
-      <c r="AC5" s="209" t="s">
+      <c r="AC5" s="208" t="s">
         <v>282</v>
       </c>
-      <c r="AD5" s="209"/>
-      <c r="AE5" s="209"/>
-      <c r="AF5" s="209"/>
-      <c r="AG5" s="209"/>
-      <c r="AH5" s="209"/>
-      <c r="AI5" s="209"/>
-      <c r="AJ5" s="209"/>
-      <c r="AK5" s="209"/>
-      <c r="AL5" s="209"/>
-      <c r="AM5" s="209"/>
+      <c r="AD5" s="208"/>
+      <c r="AE5" s="208"/>
+      <c r="AF5" s="208"/>
+      <c r="AG5" s="208"/>
+      <c r="AH5" s="208"/>
+      <c r="AI5" s="208"/>
+      <c r="AJ5" s="208"/>
+      <c r="AK5" s="208"/>
+      <c r="AL5" s="208"/>
+      <c r="AM5" s="208"/>
       <c r="AN5" s="146"/>
       <c r="AO5"/>
     </row>
@@ -13736,14 +13736,14 @@
         <v>15</v>
       </c>
       <c r="E12" s="19"/>
-      <c r="F12" s="210" t="s">
+      <c r="F12" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="210"/>
-      <c r="H12" s="210"/>
-      <c r="I12" s="210"/>
-      <c r="J12" s="210"/>
-      <c r="K12" s="210"/>
+      <c r="G12" s="209"/>
+      <c r="H12" s="209"/>
+      <c r="I12" s="209"/>
+      <c r="J12" s="209"/>
+      <c r="K12" s="209"/>
       <c r="L12" s="2"/>
       <c r="M12" s="40" t="s">
         <v>17</v>
@@ -13756,14 +13756,14 @@
         <v>15</v>
       </c>
       <c r="R12" s="19"/>
-      <c r="S12" s="210" t="s">
+      <c r="S12" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="T12" s="210"/>
-      <c r="U12" s="210"/>
-      <c r="V12" s="210"/>
-      <c r="W12" s="210"/>
-      <c r="X12" s="210"/>
+      <c r="T12" s="209"/>
+      <c r="U12" s="209"/>
+      <c r="V12" s="209"/>
+      <c r="W12" s="209"/>
+      <c r="X12" s="209"/>
       <c r="Y12" s="2"/>
       <c r="Z12" s="40" t="s">
         <v>17</v>
@@ -13776,14 +13776,14 @@
         <v>15</v>
       </c>
       <c r="AE12" s="19"/>
-      <c r="AF12" s="210" t="s">
+      <c r="AF12" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="AG12" s="210"/>
-      <c r="AH12" s="210"/>
-      <c r="AI12" s="210"/>
-      <c r="AJ12" s="210"/>
-      <c r="AK12" s="210"/>
+      <c r="AG12" s="209"/>
+      <c r="AH12" s="209"/>
+      <c r="AI12" s="209"/>
+      <c r="AJ12" s="209"/>
+      <c r="AK12" s="209"/>
       <c r="AL12" s="2"/>
       <c r="AM12" s="40" t="s">
         <v>17</v>
@@ -14543,49 +14543,49 @@
     <row r="28" spans="1:41">
       <c r="A28" s="146"/>
       <c r="B28" s="19"/>
-      <c r="C28" s="222" t="s">
+      <c r="C28" s="220" t="s">
         <v>165</v>
       </c>
-      <c r="D28" s="222"/>
-      <c r="E28" s="222"/>
-      <c r="F28" s="222"/>
-      <c r="G28" s="222"/>
-      <c r="H28" s="222"/>
-      <c r="I28" s="222"/>
-      <c r="J28" s="222"/>
-      <c r="K28" s="222"/>
-      <c r="L28" s="222"/>
-      <c r="M28" s="222"/>
+      <c r="D28" s="220"/>
+      <c r="E28" s="220"/>
+      <c r="F28" s="220"/>
+      <c r="G28" s="220"/>
+      <c r="H28" s="220"/>
+      <c r="I28" s="220"/>
+      <c r="J28" s="220"/>
+      <c r="K28" s="220"/>
+      <c r="L28" s="220"/>
+      <c r="M28" s="220"/>
       <c r="N28" s="146"/>
       <c r="O28" s="19"/>
-      <c r="P28" s="222" t="s">
+      <c r="P28" s="220" t="s">
         <v>200</v>
       </c>
-      <c r="Q28" s="222"/>
-      <c r="R28" s="222"/>
-      <c r="S28" s="222"/>
-      <c r="T28" s="222"/>
-      <c r="U28" s="222"/>
-      <c r="V28" s="222"/>
-      <c r="W28" s="222"/>
-      <c r="X28" s="222"/>
-      <c r="Y28" s="222"/>
-      <c r="Z28" s="222"/>
+      <c r="Q28" s="220"/>
+      <c r="R28" s="220"/>
+      <c r="S28" s="220"/>
+      <c r="T28" s="220"/>
+      <c r="U28" s="220"/>
+      <c r="V28" s="220"/>
+      <c r="W28" s="220"/>
+      <c r="X28" s="220"/>
+      <c r="Y28" s="220"/>
+      <c r="Z28" s="220"/>
       <c r="AA28" s="146"/>
       <c r="AB28" s="19"/>
-      <c r="AC28" s="222" t="s">
+      <c r="AC28" s="220" t="s">
         <v>258</v>
       </c>
-      <c r="AD28" s="222"/>
-      <c r="AE28" s="222"/>
-      <c r="AF28" s="222"/>
-      <c r="AG28" s="222"/>
-      <c r="AH28" s="222"/>
-      <c r="AI28" s="222"/>
-      <c r="AJ28" s="222"/>
-      <c r="AK28" s="222"/>
-      <c r="AL28" s="222"/>
-      <c r="AM28" s="222"/>
+      <c r="AD28" s="220"/>
+      <c r="AE28" s="220"/>
+      <c r="AF28" s="220"/>
+      <c r="AG28" s="220"/>
+      <c r="AH28" s="220"/>
+      <c r="AI28" s="220"/>
+      <c r="AJ28" s="220"/>
+      <c r="AK28" s="220"/>
+      <c r="AL28" s="220"/>
+      <c r="AM28" s="220"/>
       <c r="AN28" s="146"/>
       <c r="AO28" s="19"/>
     </row>
@@ -14594,34 +14594,34 @@
       <c r="B29" s="19"/>
       <c r="N29" s="146"/>
       <c r="O29" s="19"/>
-      <c r="P29" s="223" t="s">
+      <c r="P29" s="221" t="s">
         <v>279</v>
       </c>
-      <c r="Q29" s="222"/>
-      <c r="R29" s="222"/>
-      <c r="S29" s="222"/>
-      <c r="T29" s="222"/>
-      <c r="U29" s="222"/>
-      <c r="V29" s="222"/>
-      <c r="W29" s="222"/>
-      <c r="X29" s="222"/>
-      <c r="Y29" s="222"/>
-      <c r="Z29" s="222"/>
+      <c r="Q29" s="220"/>
+      <c r="R29" s="220"/>
+      <c r="S29" s="220"/>
+      <c r="T29" s="220"/>
+      <c r="U29" s="220"/>
+      <c r="V29" s="220"/>
+      <c r="W29" s="220"/>
+      <c r="X29" s="220"/>
+      <c r="Y29" s="220"/>
+      <c r="Z29" s="220"/>
       <c r="AA29" s="146"/>
       <c r="AB29" s="19"/>
-      <c r="AC29" s="222" t="s">
+      <c r="AC29" s="220" t="s">
         <v>259</v>
       </c>
-      <c r="AD29" s="222"/>
-      <c r="AE29" s="222"/>
-      <c r="AF29" s="222"/>
-      <c r="AG29" s="222"/>
-      <c r="AH29" s="222"/>
-      <c r="AI29" s="222"/>
-      <c r="AJ29" s="222"/>
-      <c r="AK29" s="222"/>
-      <c r="AL29" s="222"/>
-      <c r="AM29" s="222"/>
+      <c r="AD29" s="220"/>
+      <c r="AE29" s="220"/>
+      <c r="AF29" s="220"/>
+      <c r="AG29" s="220"/>
+      <c r="AH29" s="220"/>
+      <c r="AI29" s="220"/>
+      <c r="AJ29" s="220"/>
+      <c r="AK29" s="220"/>
+      <c r="AL29" s="220"/>
+      <c r="AM29" s="220"/>
       <c r="AN29" s="146"/>
       <c r="AO29" s="19"/>
     </row>
@@ -14630,19 +14630,19 @@
       <c r="B30" s="19"/>
       <c r="N30" s="146"/>
       <c r="O30" s="19"/>
-      <c r="P30" s="223" t="s">
+      <c r="P30" s="221" t="s">
         <v>280</v>
       </c>
-      <c r="Q30" s="222"/>
-      <c r="R30" s="222"/>
-      <c r="S30" s="222"/>
-      <c r="T30" s="222"/>
-      <c r="U30" s="222"/>
-      <c r="V30" s="222"/>
-      <c r="W30" s="222"/>
-      <c r="X30" s="222"/>
-      <c r="Y30" s="222"/>
-      <c r="Z30" s="222"/>
+      <c r="Q30" s="220"/>
+      <c r="R30" s="220"/>
+      <c r="S30" s="220"/>
+      <c r="T30" s="220"/>
+      <c r="U30" s="220"/>
+      <c r="V30" s="220"/>
+      <c r="W30" s="220"/>
+      <c r="X30" s="220"/>
+      <c r="Y30" s="220"/>
+      <c r="Z30" s="220"/>
       <c r="AA30" s="146"/>
       <c r="AB30" s="19"/>
       <c r="AN30" s="146"/>
@@ -14653,34 +14653,34 @@
       <c r="B31" s="19"/>
       <c r="N31" s="146"/>
       <c r="O31" s="19"/>
-      <c r="P31" s="222" t="s">
+      <c r="P31" s="220" t="s">
         <v>195</v>
       </c>
-      <c r="Q31" s="222"/>
-      <c r="R31" s="222"/>
-      <c r="S31" s="222"/>
-      <c r="T31" s="222"/>
-      <c r="U31" s="222"/>
-      <c r="V31" s="222"/>
-      <c r="W31" s="222"/>
-      <c r="X31" s="222"/>
-      <c r="Y31" s="222"/>
-      <c r="Z31" s="222"/>
+      <c r="Q31" s="220"/>
+      <c r="R31" s="220"/>
+      <c r="S31" s="220"/>
+      <c r="T31" s="220"/>
+      <c r="U31" s="220"/>
+      <c r="V31" s="220"/>
+      <c r="W31" s="220"/>
+      <c r="X31" s="220"/>
+      <c r="Y31" s="220"/>
+      <c r="Z31" s="220"/>
       <c r="AA31" s="146"/>
       <c r="AB31" s="19"/>
-      <c r="AC31" s="222" t="s">
+      <c r="AC31" s="220" t="s">
         <v>281</v>
       </c>
-      <c r="AD31" s="222"/>
-      <c r="AE31" s="222"/>
-      <c r="AF31" s="222"/>
-      <c r="AG31" s="222"/>
-      <c r="AH31" s="222"/>
-      <c r="AI31" s="222"/>
-      <c r="AJ31" s="222"/>
-      <c r="AK31" s="222"/>
-      <c r="AL31" s="222"/>
-      <c r="AM31" s="222"/>
+      <c r="AD31" s="220"/>
+      <c r="AE31" s="220"/>
+      <c r="AF31" s="220"/>
+      <c r="AG31" s="220"/>
+      <c r="AH31" s="220"/>
+      <c r="AI31" s="220"/>
+      <c r="AJ31" s="220"/>
+      <c r="AK31" s="220"/>
+      <c r="AL31" s="220"/>
+      <c r="AM31" s="220"/>
       <c r="AN31" s="146"/>
       <c r="AO31" s="19"/>
     </row>
@@ -14706,18 +14706,18 @@
     <row r="33" spans="1:41">
       <c r="A33" s="146"/>
       <c r="N33" s="146"/>
-      <c r="Q33" s="221" t="s">
+      <c r="Q33" s="206" t="s">
         <v>162</v>
       </c>
-      <c r="R33" s="221"/>
-      <c r="S33" s="221"/>
-      <c r="T33" s="221"/>
-      <c r="U33" s="221"/>
-      <c r="V33" s="221"/>
-      <c r="W33" s="221"/>
-      <c r="X33" s="221"/>
-      <c r="Y33" s="221"/>
-      <c r="Z33" s="221"/>
+      <c r="R33" s="206"/>
+      <c r="S33" s="206"/>
+      <c r="T33" s="206"/>
+      <c r="U33" s="206"/>
+      <c r="V33" s="206"/>
+      <c r="W33" s="206"/>
+      <c r="X33" s="206"/>
+      <c r="Y33" s="206"/>
+      <c r="Z33" s="206"/>
       <c r="AA33" s="146"/>
       <c r="AN33" s="146"/>
     </row>
@@ -14727,18 +14727,18 @@
       <c r="P34" s="115">
         <v>1</v>
       </c>
-      <c r="Q34" s="216" t="s">
+      <c r="Q34" s="219" t="s">
         <v>185</v>
       </c>
-      <c r="R34" s="216"/>
-      <c r="S34" s="216"/>
-      <c r="T34" s="216"/>
-      <c r="U34" s="216"/>
-      <c r="V34" s="216"/>
-      <c r="W34" s="216"/>
-      <c r="X34" s="216"/>
-      <c r="Y34" s="216"/>
-      <c r="Z34" s="216"/>
+      <c r="R34" s="219"/>
+      <c r="S34" s="219"/>
+      <c r="T34" s="219"/>
+      <c r="U34" s="219"/>
+      <c r="V34" s="219"/>
+      <c r="W34" s="219"/>
+      <c r="X34" s="219"/>
+      <c r="Y34" s="219"/>
+      <c r="Z34" s="219"/>
       <c r="AA34" s="146"/>
       <c r="AD34" s="141" t="s">
         <v>162</v>
@@ -14760,34 +14760,34 @@
       <c r="P35" s="115">
         <v>2</v>
       </c>
-      <c r="Q35" s="216" t="s">
+      <c r="Q35" s="219" t="s">
         <v>186</v>
       </c>
-      <c r="R35" s="216"/>
-      <c r="S35" s="216"/>
-      <c r="T35" s="216"/>
-      <c r="U35" s="216"/>
-      <c r="V35" s="216"/>
-      <c r="W35" s="216"/>
-      <c r="X35" s="216"/>
-      <c r="Y35" s="216"/>
-      <c r="Z35" s="216"/>
+      <c r="R35" s="219"/>
+      <c r="S35" s="219"/>
+      <c r="T35" s="219"/>
+      <c r="U35" s="219"/>
+      <c r="V35" s="219"/>
+      <c r="W35" s="219"/>
+      <c r="X35" s="219"/>
+      <c r="Y35" s="219"/>
+      <c r="Z35" s="219"/>
       <c r="AA35" s="146"/>
       <c r="AC35" s="115">
         <v>1</v>
       </c>
-      <c r="AD35" s="216" t="s">
+      <c r="AD35" s="219" t="s">
         <v>283</v>
       </c>
-      <c r="AE35" s="216"/>
-      <c r="AF35" s="216"/>
-      <c r="AG35" s="216"/>
-      <c r="AH35" s="216"/>
-      <c r="AI35" s="216"/>
-      <c r="AJ35" s="216"/>
-      <c r="AK35" s="216"/>
-      <c r="AL35" s="216"/>
-      <c r="AM35" s="216"/>
+      <c r="AE35" s="219"/>
+      <c r="AF35" s="219"/>
+      <c r="AG35" s="219"/>
+      <c r="AH35" s="219"/>
+      <c r="AI35" s="219"/>
+      <c r="AJ35" s="219"/>
+      <c r="AK35" s="219"/>
+      <c r="AL35" s="219"/>
+      <c r="AM35" s="219"/>
       <c r="AN35" s="146"/>
     </row>
     <row r="36" spans="1:41">
@@ -14796,34 +14796,34 @@
       <c r="P36" s="115">
         <v>3</v>
       </c>
-      <c r="Q36" s="216" t="s">
+      <c r="Q36" s="219" t="s">
         <v>188</v>
       </c>
-      <c r="R36" s="216"/>
-      <c r="S36" s="216"/>
-      <c r="T36" s="216"/>
-      <c r="U36" s="216"/>
-      <c r="V36" s="216"/>
-      <c r="W36" s="216"/>
-      <c r="X36" s="216"/>
-      <c r="Y36" s="216"/>
-      <c r="Z36" s="216"/>
+      <c r="R36" s="219"/>
+      <c r="S36" s="219"/>
+      <c r="T36" s="219"/>
+      <c r="U36" s="219"/>
+      <c r="V36" s="219"/>
+      <c r="W36" s="219"/>
+      <c r="X36" s="219"/>
+      <c r="Y36" s="219"/>
+      <c r="Z36" s="219"/>
       <c r="AA36" s="146"/>
       <c r="AC36" s="115">
         <v>2</v>
       </c>
-      <c r="AD36" s="216" t="s">
+      <c r="AD36" s="219" t="s">
         <v>284</v>
       </c>
-      <c r="AE36" s="216"/>
-      <c r="AF36" s="216"/>
-      <c r="AG36" s="216"/>
-      <c r="AH36" s="216"/>
-      <c r="AI36" s="216"/>
-      <c r="AJ36" s="216"/>
-      <c r="AK36" s="216"/>
-      <c r="AL36" s="216"/>
-      <c r="AM36" s="216"/>
+      <c r="AE36" s="219"/>
+      <c r="AF36" s="219"/>
+      <c r="AG36" s="219"/>
+      <c r="AH36" s="219"/>
+      <c r="AI36" s="219"/>
+      <c r="AJ36" s="219"/>
+      <c r="AK36" s="219"/>
+      <c r="AL36" s="219"/>
+      <c r="AM36" s="219"/>
       <c r="AN36" s="146"/>
     </row>
     <row r="37" spans="1:41">
@@ -14832,30 +14832,30 @@
       <c r="P37" s="115">
         <v>4</v>
       </c>
-      <c r="Q37" s="216" t="s">
+      <c r="Q37" s="219" t="s">
         <v>187</v>
       </c>
-      <c r="R37" s="216"/>
-      <c r="S37" s="216"/>
-      <c r="T37" s="216"/>
-      <c r="U37" s="216"/>
-      <c r="V37" s="216"/>
-      <c r="W37" s="216"/>
-      <c r="X37" s="216"/>
-      <c r="Y37" s="216"/>
-      <c r="Z37" s="216"/>
+      <c r="R37" s="219"/>
+      <c r="S37" s="219"/>
+      <c r="T37" s="219"/>
+      <c r="U37" s="219"/>
+      <c r="V37" s="219"/>
+      <c r="W37" s="219"/>
+      <c r="X37" s="219"/>
+      <c r="Y37" s="219"/>
+      <c r="Z37" s="219"/>
       <c r="AA37" s="146"/>
       <c r="AC37" s="115"/>
-      <c r="AD37" s="216"/>
-      <c r="AE37" s="216"/>
-      <c r="AF37" s="216"/>
-      <c r="AG37" s="216"/>
-      <c r="AH37" s="216"/>
-      <c r="AI37" s="216"/>
-      <c r="AJ37" s="216"/>
-      <c r="AK37" s="216"/>
-      <c r="AL37" s="216"/>
-      <c r="AM37" s="216"/>
+      <c r="AD37" s="219"/>
+      <c r="AE37" s="219"/>
+      <c r="AF37" s="219"/>
+      <c r="AG37" s="219"/>
+      <c r="AH37" s="219"/>
+      <c r="AI37" s="219"/>
+      <c r="AJ37" s="219"/>
+      <c r="AK37" s="219"/>
+      <c r="AL37" s="219"/>
+      <c r="AM37" s="219"/>
       <c r="AN37" s="146"/>
     </row>
     <row r="38" spans="1:41">
@@ -14864,18 +14864,18 @@
       <c r="P38" s="115">
         <v>5</v>
       </c>
-      <c r="Q38" s="216" t="s">
+      <c r="Q38" s="219" t="s">
         <v>189</v>
       </c>
-      <c r="R38" s="216"/>
-      <c r="S38" s="216"/>
-      <c r="T38" s="216"/>
-      <c r="U38" s="216"/>
-      <c r="V38" s="216"/>
-      <c r="W38" s="216"/>
-      <c r="X38" s="216"/>
-      <c r="Y38" s="216"/>
-      <c r="Z38" s="216"/>
+      <c r="R38" s="219"/>
+      <c r="S38" s="219"/>
+      <c r="T38" s="219"/>
+      <c r="U38" s="219"/>
+      <c r="V38" s="219"/>
+      <c r="W38" s="219"/>
+      <c r="X38" s="219"/>
+      <c r="Y38" s="219"/>
+      <c r="Z38" s="219"/>
       <c r="AA38" s="146"/>
       <c r="AN38" s="146"/>
     </row>
@@ -14885,18 +14885,18 @@
       <c r="P39" s="115">
         <v>6</v>
       </c>
-      <c r="Q39" s="216" t="s">
+      <c r="Q39" s="219" t="s">
         <v>190</v>
       </c>
-      <c r="R39" s="216"/>
-      <c r="S39" s="216"/>
-      <c r="T39" s="216"/>
-      <c r="U39" s="216"/>
-      <c r="V39" s="216"/>
-      <c r="W39" s="216"/>
-      <c r="X39" s="216"/>
-      <c r="Y39" s="216"/>
-      <c r="Z39" s="216"/>
+      <c r="R39" s="219"/>
+      <c r="S39" s="219"/>
+      <c r="T39" s="219"/>
+      <c r="U39" s="219"/>
+      <c r="V39" s="219"/>
+      <c r="W39" s="219"/>
+      <c r="X39" s="219"/>
+      <c r="Y39" s="219"/>
+      <c r="Z39" s="219"/>
       <c r="AA39" s="146"/>
       <c r="AN39" s="146"/>
     </row>
@@ -14908,30 +14908,30 @@
       <c r="P40" s="115">
         <v>7</v>
       </c>
-      <c r="Q40" s="216" t="s">
+      <c r="Q40" s="219" t="s">
         <v>191</v>
       </c>
-      <c r="R40" s="216"/>
-      <c r="S40" s="216"/>
-      <c r="T40" s="216"/>
-      <c r="U40" s="216"/>
-      <c r="V40" s="216"/>
-      <c r="W40" s="216"/>
-      <c r="X40" s="216"/>
-      <c r="Y40" s="216"/>
-      <c r="Z40" s="216"/>
+      <c r="R40" s="219"/>
+      <c r="S40" s="219"/>
+      <c r="T40" s="219"/>
+      <c r="U40" s="219"/>
+      <c r="V40" s="219"/>
+      <c r="W40" s="219"/>
+      <c r="X40" s="219"/>
+      <c r="Y40" s="219"/>
+      <c r="Z40" s="219"/>
       <c r="AA40" s="146"/>
       <c r="AB40" s="115"/>
-      <c r="AD40" s="216"/>
-      <c r="AE40" s="216"/>
-      <c r="AF40" s="216"/>
-      <c r="AG40" s="216"/>
-      <c r="AH40" s="216"/>
-      <c r="AI40" s="216"/>
-      <c r="AJ40" s="216"/>
-      <c r="AK40" s="216"/>
-      <c r="AL40" s="216"/>
-      <c r="AM40" s="216"/>
+      <c r="AD40" s="219"/>
+      <c r="AE40" s="219"/>
+      <c r="AF40" s="219"/>
+      <c r="AG40" s="219"/>
+      <c r="AH40" s="219"/>
+      <c r="AI40" s="219"/>
+      <c r="AJ40" s="219"/>
+      <c r="AK40" s="219"/>
+      <c r="AL40" s="219"/>
+      <c r="AM40" s="219"/>
       <c r="AN40" s="146"/>
       <c r="AO40" s="115"/>
     </row>
@@ -14943,30 +14943,30 @@
       <c r="P41" s="115">
         <v>8</v>
       </c>
-      <c r="Q41" s="216" t="s">
+      <c r="Q41" s="219" t="s">
         <v>192</v>
       </c>
-      <c r="R41" s="216"/>
-      <c r="S41" s="216"/>
-      <c r="T41" s="216"/>
-      <c r="U41" s="216"/>
-      <c r="V41" s="216"/>
-      <c r="W41" s="216"/>
-      <c r="X41" s="216"/>
-      <c r="Y41" s="216"/>
-      <c r="Z41" s="216"/>
+      <c r="R41" s="219"/>
+      <c r="S41" s="219"/>
+      <c r="T41" s="219"/>
+      <c r="U41" s="219"/>
+      <c r="V41" s="219"/>
+      <c r="W41" s="219"/>
+      <c r="X41" s="219"/>
+      <c r="Y41" s="219"/>
+      <c r="Z41" s="219"/>
       <c r="AA41" s="146"/>
       <c r="AB41" s="115"/>
-      <c r="AD41" s="216"/>
-      <c r="AE41" s="216"/>
-      <c r="AF41" s="216"/>
-      <c r="AG41" s="216"/>
-      <c r="AH41" s="216"/>
-      <c r="AI41" s="216"/>
-      <c r="AJ41" s="216"/>
-      <c r="AK41" s="216"/>
-      <c r="AL41" s="216"/>
-      <c r="AM41" s="216"/>
+      <c r="AD41" s="219"/>
+      <c r="AE41" s="219"/>
+      <c r="AF41" s="219"/>
+      <c r="AG41" s="219"/>
+      <c r="AH41" s="219"/>
+      <c r="AI41" s="219"/>
+      <c r="AJ41" s="219"/>
+      <c r="AK41" s="219"/>
+      <c r="AL41" s="219"/>
+      <c r="AM41" s="219"/>
       <c r="AN41" s="146"/>
       <c r="AO41" s="115"/>
     </row>
@@ -15142,6 +15142,27 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="AD41:AM41"/>
+    <mergeCell ref="AD37:AM37"/>
+    <mergeCell ref="AD35:AM35"/>
+    <mergeCell ref="AD36:AM36"/>
+    <mergeCell ref="AD40:AM40"/>
+    <mergeCell ref="AC31:AM31"/>
+    <mergeCell ref="AC3:AM3"/>
+    <mergeCell ref="AC5:AM5"/>
+    <mergeCell ref="AF12:AK12"/>
+    <mergeCell ref="AC28:AM28"/>
+    <mergeCell ref="AC29:AM29"/>
+    <mergeCell ref="C28:M28"/>
+    <mergeCell ref="P30:Z30"/>
+    <mergeCell ref="P28:Z28"/>
+    <mergeCell ref="P29:Z29"/>
+    <mergeCell ref="C3:M3"/>
+    <mergeCell ref="P3:Z3"/>
+    <mergeCell ref="C5:M5"/>
+    <mergeCell ref="P5:Z5"/>
+    <mergeCell ref="F12:K12"/>
+    <mergeCell ref="S12:X12"/>
     <mergeCell ref="Q40:Z40"/>
     <mergeCell ref="Q41:Z41"/>
     <mergeCell ref="Q37:Z37"/>
@@ -15152,27 +15173,6 @@
     <mergeCell ref="Q34:Z34"/>
     <mergeCell ref="Q35:Z35"/>
     <mergeCell ref="Q36:Z36"/>
-    <mergeCell ref="C28:M28"/>
-    <mergeCell ref="P30:Z30"/>
-    <mergeCell ref="P28:Z28"/>
-    <mergeCell ref="P29:Z29"/>
-    <mergeCell ref="C3:M3"/>
-    <mergeCell ref="P3:Z3"/>
-    <mergeCell ref="C5:M5"/>
-    <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="F12:K12"/>
-    <mergeCell ref="S12:X12"/>
-    <mergeCell ref="AC31:AM31"/>
-    <mergeCell ref="AC3:AM3"/>
-    <mergeCell ref="AC5:AM5"/>
-    <mergeCell ref="AF12:AK12"/>
-    <mergeCell ref="AC28:AM28"/>
-    <mergeCell ref="AC29:AM29"/>
-    <mergeCell ref="AD41:AM41"/>
-    <mergeCell ref="AD37:AM37"/>
-    <mergeCell ref="AD35:AM35"/>
-    <mergeCell ref="AD36:AM36"/>
-    <mergeCell ref="AD40:AM40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="55" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
@@ -15246,34 +15246,34 @@
     <row r="3" spans="1:28" s="74" customFormat="1" ht="19">
       <c r="A3" s="146"/>
       <c r="B3"/>
-      <c r="C3" s="217" t="s">
+      <c r="C3" s="210" t="s">
         <v>177</v>
       </c>
-      <c r="D3" s="217"/>
-      <c r="E3" s="217"/>
-      <c r="F3" s="217"/>
-      <c r="G3" s="217"/>
-      <c r="H3" s="217"/>
-      <c r="I3" s="217"/>
-      <c r="J3" s="217"/>
-      <c r="K3" s="217"/>
-      <c r="L3" s="217"/>
-      <c r="M3" s="217"/>
+      <c r="D3" s="210"/>
+      <c r="E3" s="210"/>
+      <c r="F3" s="210"/>
+      <c r="G3" s="210"/>
+      <c r="H3" s="210"/>
+      <c r="I3" s="210"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="210"/>
+      <c r="M3" s="210"/>
       <c r="N3" s="146"/>
       <c r="O3"/>
-      <c r="P3" s="217" t="s">
+      <c r="P3" s="210" t="s">
         <v>178</v>
       </c>
-      <c r="Q3" s="217"/>
-      <c r="R3" s="217"/>
-      <c r="S3" s="217"/>
-      <c r="T3" s="217"/>
-      <c r="U3" s="217"/>
-      <c r="V3" s="217"/>
-      <c r="W3" s="217"/>
-      <c r="X3" s="217"/>
-      <c r="Y3" s="217"/>
-      <c r="Z3" s="217"/>
+      <c r="Q3" s="210"/>
+      <c r="R3" s="210"/>
+      <c r="S3" s="210"/>
+      <c r="T3" s="210"/>
+      <c r="U3" s="210"/>
+      <c r="V3" s="210"/>
+      <c r="W3" s="210"/>
+      <c r="X3" s="210"/>
+      <c r="Y3" s="210"/>
+      <c r="Z3" s="210"/>
       <c r="AA3" s="146"/>
       <c r="AB3"/>
     </row>
@@ -15448,14 +15448,14 @@
       <c r="D10" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="211" t="s">
+      <c r="F10" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="211"/>
-      <c r="H10" s="211"/>
-      <c r="I10" s="211"/>
-      <c r="J10" s="211"/>
-      <c r="K10" s="211"/>
+      <c r="G10" s="214"/>
+      <c r="H10" s="214"/>
+      <c r="I10" s="214"/>
+      <c r="J10" s="214"/>
+      <c r="K10" s="214"/>
       <c r="M10" s="4" t="s">
         <v>17</v>
       </c>
@@ -15467,14 +15467,14 @@
         <v>15</v>
       </c>
       <c r="R10" s="1"/>
-      <c r="S10" s="211" t="s">
+      <c r="S10" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="T10" s="211"/>
-      <c r="U10" s="211"/>
-      <c r="V10" s="211"/>
-      <c r="W10" s="211"/>
-      <c r="X10" s="211"/>
+      <c r="T10" s="214"/>
+      <c r="U10" s="214"/>
+      <c r="V10" s="214"/>
+      <c r="W10" s="214"/>
+      <c r="X10" s="214"/>
       <c r="Y10" s="19"/>
       <c r="Z10" s="4" t="s">
         <v>17</v>
@@ -16612,105 +16612,105 @@
     <row r="43" spans="1:28">
       <c r="A43" s="146"/>
       <c r="B43" s="115"/>
-      <c r="D43" s="221" t="s">
+      <c r="D43" s="206" t="s">
         <v>162</v>
       </c>
-      <c r="E43" s="221"/>
-      <c r="F43" s="221"/>
-      <c r="G43" s="221"/>
-      <c r="H43" s="221"/>
-      <c r="I43" s="221"/>
-      <c r="J43" s="221"/>
-      <c r="K43" s="221"/>
-      <c r="L43" s="221"/>
-      <c r="M43" s="221"/>
+      <c r="E43" s="206"/>
+      <c r="F43" s="206"/>
+      <c r="G43" s="206"/>
+      <c r="H43" s="206"/>
+      <c r="I43" s="206"/>
+      <c r="J43" s="206"/>
+      <c r="K43" s="206"/>
+      <c r="L43" s="206"/>
+      <c r="M43" s="206"/>
       <c r="N43" s="146"/>
       <c r="O43" s="115"/>
       <c r="P43" s="115"/>
-      <c r="Q43" s="221" t="s">
+      <c r="Q43" s="206" t="s">
         <v>162</v>
       </c>
-      <c r="R43" s="221"/>
-      <c r="S43" s="221"/>
-      <c r="T43" s="221"/>
-      <c r="U43" s="221"/>
-      <c r="V43" s="221"/>
-      <c r="W43" s="221"/>
-      <c r="X43" s="221"/>
-      <c r="Y43" s="221"/>
-      <c r="Z43" s="221"/>
+      <c r="R43" s="206"/>
+      <c r="S43" s="206"/>
+      <c r="T43" s="206"/>
+      <c r="U43" s="206"/>
+      <c r="V43" s="206"/>
+      <c r="W43" s="206"/>
+      <c r="X43" s="206"/>
+      <c r="Y43" s="206"/>
+      <c r="Z43" s="206"/>
       <c r="AA43" s="146"/>
       <c r="AB43" s="115"/>
     </row>
     <row r="44" spans="1:28">
       <c r="A44" s="146"/>
       <c r="B44" s="115"/>
-      <c r="C44" s="216" t="s">
+      <c r="C44" s="219" t="s">
         <v>164</v>
       </c>
-      <c r="D44" s="216"/>
-      <c r="E44" s="216"/>
-      <c r="F44" s="216"/>
-      <c r="G44" s="216"/>
-      <c r="H44" s="216"/>
-      <c r="I44" s="216"/>
-      <c r="J44" s="216"/>
-      <c r="K44" s="216"/>
-      <c r="L44" s="216"/>
-      <c r="M44" s="216"/>
+      <c r="D44" s="219"/>
+      <c r="E44" s="219"/>
+      <c r="F44" s="219"/>
+      <c r="G44" s="219"/>
+      <c r="H44" s="219"/>
+      <c r="I44" s="219"/>
+      <c r="J44" s="219"/>
+      <c r="K44" s="219"/>
+      <c r="L44" s="219"/>
+      <c r="M44" s="219"/>
       <c r="N44" s="146"/>
       <c r="O44" s="115"/>
       <c r="P44" s="115">
         <v>1</v>
       </c>
-      <c r="Q44" s="216" t="s">
+      <c r="Q44" s="219" t="s">
         <v>173</v>
       </c>
-      <c r="R44" s="216"/>
-      <c r="S44" s="216"/>
-      <c r="T44" s="216"/>
-      <c r="U44" s="216"/>
-      <c r="V44" s="216"/>
-      <c r="W44" s="216"/>
-      <c r="X44" s="216"/>
-      <c r="Y44" s="216"/>
-      <c r="Z44" s="216"/>
+      <c r="R44" s="219"/>
+      <c r="S44" s="219"/>
+      <c r="T44" s="219"/>
+      <c r="U44" s="219"/>
+      <c r="V44" s="219"/>
+      <c r="W44" s="219"/>
+      <c r="X44" s="219"/>
+      <c r="Y44" s="219"/>
+      <c r="Z44" s="219"/>
       <c r="AA44" s="146"/>
       <c r="AB44" s="115"/>
     </row>
     <row r="45" spans="1:28">
       <c r="A45" s="146"/>
       <c r="B45" s="115"/>
-      <c r="C45" s="216" t="s">
+      <c r="C45" s="219" t="s">
         <v>163</v>
       </c>
-      <c r="D45" s="216"/>
-      <c r="E45" s="216"/>
-      <c r="F45" s="216"/>
-      <c r="G45" s="216"/>
-      <c r="H45" s="216"/>
-      <c r="I45" s="216"/>
-      <c r="J45" s="216"/>
-      <c r="K45" s="216"/>
-      <c r="L45" s="216"/>
-      <c r="M45" s="216"/>
+      <c r="D45" s="219"/>
+      <c r="E45" s="219"/>
+      <c r="F45" s="219"/>
+      <c r="G45" s="219"/>
+      <c r="H45" s="219"/>
+      <c r="I45" s="219"/>
+      <c r="J45" s="219"/>
+      <c r="K45" s="219"/>
+      <c r="L45" s="219"/>
+      <c r="M45" s="219"/>
       <c r="N45" s="146"/>
       <c r="O45" s="115"/>
       <c r="P45" s="115">
         <v>2</v>
       </c>
-      <c r="Q45" s="216" t="s">
+      <c r="Q45" s="219" t="s">
         <v>174</v>
       </c>
-      <c r="R45" s="216"/>
-      <c r="S45" s="216"/>
-      <c r="T45" s="216"/>
-      <c r="U45" s="216"/>
-      <c r="V45" s="216"/>
-      <c r="W45" s="216"/>
-      <c r="X45" s="216"/>
-      <c r="Y45" s="216"/>
-      <c r="Z45" s="216"/>
+      <c r="R45" s="219"/>
+      <c r="S45" s="219"/>
+      <c r="T45" s="219"/>
+      <c r="U45" s="219"/>
+      <c r="V45" s="219"/>
+      <c r="W45" s="219"/>
+      <c r="X45" s="219"/>
+      <c r="Y45" s="219"/>
+      <c r="Z45" s="219"/>
       <c r="AA45" s="146"/>
       <c r="AB45" s="115"/>
     </row>
@@ -16733,18 +16733,18 @@
       <c r="P46" s="115">
         <v>3</v>
       </c>
-      <c r="Q46" s="216" t="s">
+      <c r="Q46" s="219" t="s">
         <v>175</v>
       </c>
-      <c r="R46" s="216"/>
-      <c r="S46" s="216"/>
-      <c r="T46" s="216"/>
-      <c r="U46" s="216"/>
-      <c r="V46" s="216"/>
-      <c r="W46" s="216"/>
-      <c r="X46" s="216"/>
-      <c r="Y46" s="216"/>
-      <c r="Z46" s="216"/>
+      <c r="R46" s="219"/>
+      <c r="S46" s="219"/>
+      <c r="T46" s="219"/>
+      <c r="U46" s="219"/>
+      <c r="V46" s="219"/>
+      <c r="W46" s="219"/>
+      <c r="X46" s="219"/>
+      <c r="Y46" s="219"/>
+      <c r="Z46" s="219"/>
       <c r="AA46" s="146"/>
       <c r="AB46" s="115"/>
     </row>
@@ -16811,68 +16811,68 @@
     <row r="49" spans="1:28" ht="19">
       <c r="A49" s="146"/>
       <c r="B49" s="115"/>
-      <c r="C49" s="224" t="s">
+      <c r="C49" s="222" t="s">
         <v>24</v>
       </c>
-      <c r="D49" s="225"/>
-      <c r="E49" s="225"/>
-      <c r="F49" s="225"/>
-      <c r="G49" s="225"/>
-      <c r="H49" s="225"/>
-      <c r="I49" s="225"/>
-      <c r="J49" s="225"/>
-      <c r="K49" s="225"/>
-      <c r="L49" s="225"/>
-      <c r="M49" s="225"/>
+      <c r="D49" s="223"/>
+      <c r="E49" s="223"/>
+      <c r="F49" s="223"/>
+      <c r="G49" s="223"/>
+      <c r="H49" s="223"/>
+      <c r="I49" s="223"/>
+      <c r="J49" s="223"/>
+      <c r="K49" s="223"/>
+      <c r="L49" s="223"/>
+      <c r="M49" s="223"/>
       <c r="N49" s="146"/>
       <c r="O49" s="115"/>
-      <c r="P49" s="224" t="s">
+      <c r="P49" s="222" t="s">
         <v>24</v>
       </c>
-      <c r="Q49" s="225"/>
-      <c r="R49" s="225"/>
-      <c r="S49" s="225"/>
-      <c r="T49" s="225"/>
-      <c r="U49" s="225"/>
-      <c r="V49" s="225"/>
-      <c r="W49" s="225"/>
-      <c r="X49" s="225"/>
-      <c r="Y49" s="225"/>
-      <c r="Z49" s="225"/>
+      <c r="Q49" s="223"/>
+      <c r="R49" s="223"/>
+      <c r="S49" s="223"/>
+      <c r="T49" s="223"/>
+      <c r="U49" s="223"/>
+      <c r="V49" s="223"/>
+      <c r="W49" s="223"/>
+      <c r="X49" s="223"/>
+      <c r="Y49" s="223"/>
+      <c r="Z49" s="223"/>
       <c r="AA49" s="146"/>
       <c r="AB49" s="115"/>
     </row>
     <row r="50" spans="1:28">
       <c r="A50" s="146"/>
       <c r="B50" s="115"/>
-      <c r="C50" s="226" t="s">
+      <c r="C50" s="224" t="s">
         <v>176</v>
       </c>
-      <c r="D50" s="226"/>
-      <c r="E50" s="226"/>
-      <c r="F50" s="226"/>
-      <c r="G50" s="226"/>
-      <c r="H50" s="226"/>
-      <c r="I50" s="226"/>
-      <c r="J50" s="226"/>
-      <c r="K50" s="226"/>
-      <c r="L50" s="226"/>
-      <c r="M50" s="226"/>
+      <c r="D50" s="224"/>
+      <c r="E50" s="224"/>
+      <c r="F50" s="224"/>
+      <c r="G50" s="224"/>
+      <c r="H50" s="224"/>
+      <c r="I50" s="224"/>
+      <c r="J50" s="224"/>
+      <c r="K50" s="224"/>
+      <c r="L50" s="224"/>
+      <c r="M50" s="224"/>
       <c r="N50" s="146"/>
       <c r="O50" s="115"/>
-      <c r="P50" s="226" t="s">
+      <c r="P50" s="224" t="s">
         <v>176</v>
       </c>
-      <c r="Q50" s="226"/>
-      <c r="R50" s="226"/>
-      <c r="S50" s="226"/>
-      <c r="T50" s="226"/>
-      <c r="U50" s="226"/>
-      <c r="V50" s="226"/>
-      <c r="W50" s="226"/>
-      <c r="X50" s="226"/>
-      <c r="Y50" s="226"/>
-      <c r="Z50" s="226"/>
+      <c r="Q50" s="224"/>
+      <c r="R50" s="224"/>
+      <c r="S50" s="224"/>
+      <c r="T50" s="224"/>
+      <c r="U50" s="224"/>
+      <c r="V50" s="224"/>
+      <c r="W50" s="224"/>
+      <c r="X50" s="224"/>
+      <c r="Y50" s="224"/>
+      <c r="Z50" s="224"/>
       <c r="AA50" s="146"/>
       <c r="AB50" s="115"/>
     </row>
@@ -17633,13 +17633,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="P49:Z49"/>
-    <mergeCell ref="P50:Z50"/>
-    <mergeCell ref="Q46:Z46"/>
-    <mergeCell ref="D43:M43"/>
-    <mergeCell ref="Q43:Z43"/>
-    <mergeCell ref="C49:M49"/>
-    <mergeCell ref="C50:M50"/>
     <mergeCell ref="P3:Z3"/>
     <mergeCell ref="S10:X10"/>
     <mergeCell ref="Q44:Z44"/>
@@ -17648,6 +17641,13 @@
     <mergeCell ref="F10:K10"/>
     <mergeCell ref="C44:M44"/>
     <mergeCell ref="C45:M45"/>
+    <mergeCell ref="P49:Z49"/>
+    <mergeCell ref="P50:Z50"/>
+    <mergeCell ref="Q46:Z46"/>
+    <mergeCell ref="D43:M43"/>
+    <mergeCell ref="Q43:Z43"/>
+    <mergeCell ref="C49:M49"/>
+    <mergeCell ref="C50:M50"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C50" r:id="rId1" xr:uid="{6A2FBA32-435B-1E43-9BF4-78C6F73A13DE}"/>
@@ -17730,34 +17730,34 @@
     <row r="3" spans="1:28" s="73" customFormat="1" ht="18">
       <c r="A3" s="146"/>
       <c r="B3"/>
-      <c r="C3" s="217" t="s">
+      <c r="C3" s="210" t="s">
         <v>294</v>
       </c>
-      <c r="D3" s="217"/>
-      <c r="E3" s="217"/>
-      <c r="F3" s="217"/>
-      <c r="G3" s="217"/>
-      <c r="H3" s="217"/>
-      <c r="I3" s="217"/>
-      <c r="J3" s="217"/>
-      <c r="K3" s="217"/>
-      <c r="L3" s="217"/>
-      <c r="M3" s="217"/>
+      <c r="D3" s="210"/>
+      <c r="E3" s="210"/>
+      <c r="F3" s="210"/>
+      <c r="G3" s="210"/>
+      <c r="H3" s="210"/>
+      <c r="I3" s="210"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="210"/>
+      <c r="M3" s="210"/>
       <c r="N3" s="146"/>
       <c r="O3"/>
-      <c r="P3" s="217" t="s">
+      <c r="P3" s="210" t="s">
         <v>295</v>
       </c>
-      <c r="Q3" s="217"/>
-      <c r="R3" s="217"/>
-      <c r="S3" s="217"/>
-      <c r="T3" s="217"/>
-      <c r="U3" s="217"/>
-      <c r="V3" s="217"/>
-      <c r="W3" s="217"/>
-      <c r="X3" s="217"/>
-      <c r="Y3" s="217"/>
-      <c r="Z3" s="217"/>
+      <c r="Q3" s="210"/>
+      <c r="R3" s="210"/>
+      <c r="S3" s="210"/>
+      <c r="T3" s="210"/>
+      <c r="U3" s="210"/>
+      <c r="V3" s="210"/>
+      <c r="W3" s="210"/>
+      <c r="X3" s="210"/>
+      <c r="Y3" s="210"/>
+      <c r="Z3" s="210"/>
       <c r="AA3" s="146"/>
       <c r="AB3"/>
     </row>
@@ -17918,14 +17918,14 @@
       <c r="D10" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="211" t="s">
+      <c r="F10" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="211"/>
-      <c r="H10" s="211"/>
-      <c r="I10" s="211"/>
-      <c r="J10" s="211"/>
-      <c r="K10" s="211"/>
+      <c r="G10" s="214"/>
+      <c r="H10" s="214"/>
+      <c r="I10" s="214"/>
+      <c r="J10" s="214"/>
+      <c r="K10" s="214"/>
       <c r="M10" s="4" t="s">
         <v>17</v>
       </c>
@@ -17937,14 +17937,14 @@
         <v>15</v>
       </c>
       <c r="R10" s="19"/>
-      <c r="S10" s="211" t="s">
+      <c r="S10" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="T10" s="211"/>
-      <c r="U10" s="211"/>
-      <c r="V10" s="211"/>
-      <c r="W10" s="211"/>
-      <c r="X10" s="211"/>
+      <c r="T10" s="214"/>
+      <c r="U10" s="214"/>
+      <c r="V10" s="214"/>
+      <c r="W10" s="214"/>
+      <c r="X10" s="214"/>
       <c r="Y10" s="19"/>
       <c r="Z10" s="4" t="s">
         <v>17</v>
@@ -18447,18 +18447,18 @@
       <c r="A26" s="146"/>
       <c r="B26" s="19"/>
       <c r="C26" s="73"/>
-      <c r="D26" s="227" t="s">
+      <c r="D26" s="225" t="s">
         <v>24</v>
       </c>
-      <c r="E26" s="227"/>
-      <c r="F26" s="227"/>
-      <c r="G26" s="227"/>
-      <c r="H26" s="227"/>
-      <c r="I26" s="227"/>
-      <c r="J26" s="227"/>
-      <c r="K26" s="227"/>
-      <c r="L26" s="227"/>
-      <c r="M26" s="227"/>
+      <c r="E26" s="225"/>
+      <c r="F26" s="225"/>
+      <c r="G26" s="225"/>
+      <c r="H26" s="225"/>
+      <c r="I26" s="225"/>
+      <c r="J26" s="225"/>
+      <c r="K26" s="225"/>
+      <c r="L26" s="225"/>
+      <c r="M26" s="225"/>
       <c r="N26" s="146"/>
       <c r="O26" s="19"/>
       <c r="Q26" s="31" t="s">
@@ -18508,19 +18508,19 @@
       <c r="D29" s="49"/>
       <c r="N29" s="146"/>
       <c r="O29" s="19"/>
-      <c r="P29" s="216" t="s">
+      <c r="P29" s="219" t="s">
         <v>275</v>
       </c>
-      <c r="Q29" s="216"/>
-      <c r="R29" s="216"/>
-      <c r="S29" s="216"/>
-      <c r="T29" s="216"/>
-      <c r="U29" s="216"/>
-      <c r="V29" s="216"/>
-      <c r="W29" s="216"/>
-      <c r="X29" s="216"/>
-      <c r="Y29" s="216"/>
-      <c r="Z29" s="216"/>
+      <c r="Q29" s="219"/>
+      <c r="R29" s="219"/>
+      <c r="S29" s="219"/>
+      <c r="T29" s="219"/>
+      <c r="U29" s="219"/>
+      <c r="V29" s="219"/>
+      <c r="W29" s="219"/>
+      <c r="X29" s="219"/>
+      <c r="Y29" s="219"/>
+      <c r="Z29" s="219"/>
       <c r="AA29" s="146"/>
       <c r="AB29" s="19"/>
     </row>
@@ -18532,19 +18532,19 @@
       </c>
       <c r="N30" s="146"/>
       <c r="O30" s="19"/>
-      <c r="P30" s="216" t="s">
+      <c r="P30" s="219" t="s">
         <v>193</v>
       </c>
-      <c r="Q30" s="216"/>
-      <c r="R30" s="216"/>
-      <c r="S30" s="216"/>
-      <c r="T30" s="216"/>
-      <c r="U30" s="216"/>
-      <c r="V30" s="216"/>
-      <c r="W30" s="216"/>
-      <c r="X30" s="216"/>
-      <c r="Y30" s="216"/>
-      <c r="Z30" s="216"/>
+      <c r="Q30" s="219"/>
+      <c r="R30" s="219"/>
+      <c r="S30" s="219"/>
+      <c r="T30" s="219"/>
+      <c r="U30" s="219"/>
+      <c r="V30" s="219"/>
+      <c r="W30" s="219"/>
+      <c r="X30" s="219"/>
+      <c r="Y30" s="219"/>
+      <c r="Z30" s="219"/>
       <c r="AA30" s="146"/>
       <c r="AB30" s="19"/>
     </row>
@@ -18598,18 +18598,18 @@
       </c>
       <c r="N34" s="146"/>
       <c r="P34" s="96"/>
-      <c r="Q34" s="221" t="s">
+      <c r="Q34" s="206" t="s">
         <v>162</v>
       </c>
-      <c r="R34" s="221"/>
-      <c r="S34" s="221"/>
-      <c r="T34" s="221"/>
-      <c r="U34" s="221"/>
-      <c r="V34" s="221"/>
-      <c r="W34" s="221"/>
-      <c r="X34" s="221"/>
-      <c r="Y34" s="221"/>
-      <c r="Z34" s="221"/>
+      <c r="R34" s="206"/>
+      <c r="S34" s="206"/>
+      <c r="T34" s="206"/>
+      <c r="U34" s="206"/>
+      <c r="V34" s="206"/>
+      <c r="W34" s="206"/>
+      <c r="X34" s="206"/>
+      <c r="Y34" s="206"/>
+      <c r="Z34" s="206"/>
       <c r="AA34" s="146"/>
     </row>
     <row r="35" spans="1:28">
@@ -18624,18 +18624,18 @@
       <c r="P35" s="90">
         <v>1</v>
       </c>
-      <c r="Q35" s="216" t="s">
+      <c r="Q35" s="219" t="s">
         <v>181</v>
       </c>
-      <c r="R35" s="216"/>
-      <c r="S35" s="216"/>
-      <c r="T35" s="216"/>
-      <c r="U35" s="216"/>
-      <c r="V35" s="216"/>
-      <c r="W35" s="216"/>
-      <c r="X35" s="216"/>
-      <c r="Y35" s="216"/>
-      <c r="Z35" s="216"/>
+      <c r="R35" s="219"/>
+      <c r="S35" s="219"/>
+      <c r="T35" s="219"/>
+      <c r="U35" s="219"/>
+      <c r="V35" s="219"/>
+      <c r="W35" s="219"/>
+      <c r="X35" s="219"/>
+      <c r="Y35" s="219"/>
+      <c r="Z35" s="219"/>
       <c r="AA35" s="146"/>
     </row>
     <row r="36" spans="1:28">
@@ -18661,18 +18661,18 @@
       <c r="D37" s="169"/>
       <c r="N37" s="146"/>
       <c r="P37" s="73"/>
-      <c r="Q37" s="227" t="s">
+      <c r="Q37" s="225" t="s">
         <v>24</v>
       </c>
-      <c r="R37" s="227"/>
-      <c r="S37" s="227"/>
-      <c r="T37" s="227"/>
-      <c r="U37" s="227"/>
-      <c r="V37" s="227"/>
-      <c r="W37" s="227"/>
-      <c r="X37" s="227"/>
-      <c r="Y37" s="227"/>
-      <c r="Z37" s="227"/>
+      <c r="R37" s="225"/>
+      <c r="S37" s="225"/>
+      <c r="T37" s="225"/>
+      <c r="U37" s="225"/>
+      <c r="V37" s="225"/>
+      <c r="W37" s="225"/>
+      <c r="X37" s="225"/>
+      <c r="Y37" s="225"/>
+      <c r="Z37" s="225"/>
       <c r="AA37" s="146"/>
     </row>
     <row r="38" spans="1:28" ht="17">
@@ -19320,34 +19320,34 @@
     <row r="3" spans="1:28" s="73" customFormat="1" ht="18">
       <c r="A3" s="146"/>
       <c r="B3"/>
-      <c r="C3" s="217" t="s">
+      <c r="C3" s="210" t="s">
         <v>179</v>
       </c>
-      <c r="D3" s="217"/>
-      <c r="E3" s="217"/>
-      <c r="F3" s="217"/>
-      <c r="G3" s="217"/>
-      <c r="H3" s="217"/>
-      <c r="I3" s="217"/>
-      <c r="J3" s="217"/>
-      <c r="K3" s="217"/>
-      <c r="L3" s="217"/>
-      <c r="M3" s="217"/>
+      <c r="D3" s="210"/>
+      <c r="E3" s="210"/>
+      <c r="F3" s="210"/>
+      <c r="G3" s="210"/>
+      <c r="H3" s="210"/>
+      <c r="I3" s="210"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="210"/>
+      <c r="M3" s="210"/>
       <c r="N3" s="146"/>
       <c r="O3"/>
-      <c r="P3" s="217" t="s">
+      <c r="P3" s="210" t="s">
         <v>180</v>
       </c>
-      <c r="Q3" s="217"/>
-      <c r="R3" s="217"/>
-      <c r="S3" s="217"/>
-      <c r="T3" s="217"/>
-      <c r="U3" s="217"/>
-      <c r="V3" s="217"/>
-      <c r="W3" s="217"/>
-      <c r="X3" s="217"/>
-      <c r="Y3" s="217"/>
-      <c r="Z3" s="217"/>
+      <c r="Q3" s="210"/>
+      <c r="R3" s="210"/>
+      <c r="S3" s="210"/>
+      <c r="T3" s="210"/>
+      <c r="U3" s="210"/>
+      <c r="V3" s="210"/>
+      <c r="W3" s="210"/>
+      <c r="X3" s="210"/>
+      <c r="Y3" s="210"/>
+      <c r="Z3" s="210"/>
       <c r="AA3" s="146"/>
       <c r="AB3"/>
     </row>
@@ -19512,14 +19512,14 @@
       <c r="D10" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="211" t="s">
+      <c r="F10" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="211"/>
-      <c r="H10" s="211"/>
-      <c r="I10" s="211"/>
-      <c r="J10" s="211"/>
-      <c r="K10" s="211"/>
+      <c r="G10" s="214"/>
+      <c r="H10" s="214"/>
+      <c r="I10" s="214"/>
+      <c r="J10" s="214"/>
+      <c r="K10" s="214"/>
       <c r="M10" s="4" t="s">
         <v>17</v>
       </c>
@@ -19530,14 +19530,14 @@
       <c r="Q10" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S10" s="211" t="s">
+      <c r="S10" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="T10" s="211"/>
-      <c r="U10" s="211"/>
-      <c r="V10" s="211"/>
-      <c r="W10" s="211"/>
-      <c r="X10" s="211"/>
+      <c r="T10" s="214"/>
+      <c r="U10" s="214"/>
+      <c r="V10" s="214"/>
+      <c r="W10" s="214"/>
+      <c r="X10" s="214"/>
       <c r="Z10" s="166" t="s">
         <v>17</v>
       </c>
@@ -20067,64 +20067,64 @@
     <row r="29" spans="1:28" ht="19">
       <c r="A29" s="146"/>
       <c r="B29" s="19"/>
-      <c r="D29" s="207" t="s">
+      <c r="D29" s="227" t="s">
         <v>24</v>
       </c>
-      <c r="E29" s="208"/>
-      <c r="F29" s="208"/>
-      <c r="G29" s="208"/>
-      <c r="H29" s="208"/>
-      <c r="I29" s="208"/>
-      <c r="J29" s="208"/>
-      <c r="K29" s="208"/>
-      <c r="L29" s="208"/>
-      <c r="M29" s="208"/>
+      <c r="E29" s="228"/>
+      <c r="F29" s="228"/>
+      <c r="G29" s="228"/>
+      <c r="H29" s="228"/>
+      <c r="I29" s="228"/>
+      <c r="J29" s="228"/>
+      <c r="K29" s="228"/>
+      <c r="L29" s="228"/>
+      <c r="M29" s="228"/>
       <c r="N29" s="146"/>
       <c r="O29" s="19"/>
-      <c r="Q29" s="207" t="s">
+      <c r="Q29" s="227" t="s">
         <v>24</v>
       </c>
-      <c r="R29" s="208"/>
-      <c r="S29" s="208"/>
-      <c r="T29" s="208"/>
-      <c r="U29" s="208"/>
-      <c r="V29" s="208"/>
-      <c r="W29" s="208"/>
-      <c r="X29" s="208"/>
-      <c r="Y29" s="208"/>
-      <c r="Z29" s="208"/>
+      <c r="R29" s="228"/>
+      <c r="S29" s="228"/>
+      <c r="T29" s="228"/>
+      <c r="U29" s="228"/>
+      <c r="V29" s="228"/>
+      <c r="W29" s="228"/>
+      <c r="X29" s="228"/>
+      <c r="Y29" s="228"/>
+      <c r="Z29" s="228"/>
       <c r="AA29" s="146"/>
       <c r="AB29" s="19"/>
     </row>
     <row r="30" spans="1:28">
       <c r="A30" s="146"/>
       <c r="B30" s="19"/>
-      <c r="D30" s="206" t="s">
+      <c r="D30" s="226" t="s">
         <v>176</v>
       </c>
-      <c r="E30" s="206"/>
-      <c r="F30" s="206"/>
-      <c r="G30" s="206"/>
-      <c r="H30" s="206"/>
-      <c r="I30" s="206"/>
-      <c r="J30" s="206"/>
-      <c r="K30" s="206"/>
-      <c r="L30" s="206"/>
-      <c r="M30" s="206"/>
+      <c r="E30" s="226"/>
+      <c r="F30" s="226"/>
+      <c r="G30" s="226"/>
+      <c r="H30" s="226"/>
+      <c r="I30" s="226"/>
+      <c r="J30" s="226"/>
+      <c r="K30" s="226"/>
+      <c r="L30" s="226"/>
+      <c r="M30" s="226"/>
       <c r="N30" s="146"/>
       <c r="O30" s="19"/>
-      <c r="Q30" s="206" t="s">
+      <c r="Q30" s="226" t="s">
         <v>176</v>
       </c>
-      <c r="R30" s="206"/>
-      <c r="S30" s="206"/>
-      <c r="T30" s="206"/>
-      <c r="U30" s="206"/>
-      <c r="V30" s="206"/>
-      <c r="W30" s="206"/>
-      <c r="X30" s="206"/>
-      <c r="Y30" s="206"/>
-      <c r="Z30" s="206"/>
+      <c r="R30" s="226"/>
+      <c r="S30" s="226"/>
+      <c r="T30" s="226"/>
+      <c r="U30" s="226"/>
+      <c r="V30" s="226"/>
+      <c r="W30" s="226"/>
+      <c r="X30" s="226"/>
+      <c r="Y30" s="226"/>
+      <c r="Z30" s="226"/>
       <c r="AA30" s="146"/>
       <c r="AB30" s="19"/>
     </row>
@@ -21409,49 +21409,49 @@
     <row r="3" spans="1:41" s="74" customFormat="1" ht="19">
       <c r="A3" s="146"/>
       <c r="B3"/>
-      <c r="C3" s="209" t="s">
+      <c r="C3" s="208" t="s">
         <v>182</v>
       </c>
-      <c r="D3" s="209"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="209"/>
-      <c r="G3" s="209"/>
-      <c r="H3" s="209"/>
-      <c r="I3" s="209"/>
-      <c r="J3" s="209"/>
-      <c r="K3" s="209"/>
-      <c r="L3" s="209"/>
-      <c r="M3" s="209"/>
+      <c r="D3" s="208"/>
+      <c r="E3" s="208"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="208"/>
+      <c r="H3" s="208"/>
+      <c r="I3" s="208"/>
+      <c r="J3" s="208"/>
+      <c r="K3" s="208"/>
+      <c r="L3" s="208"/>
+      <c r="M3" s="208"/>
       <c r="N3" s="146"/>
       <c r="O3"/>
-      <c r="P3" s="209" t="s">
+      <c r="P3" s="208" t="s">
         <v>183</v>
       </c>
-      <c r="Q3" s="209"/>
-      <c r="R3" s="209"/>
-      <c r="S3" s="209"/>
-      <c r="T3" s="209"/>
-      <c r="U3" s="209"/>
-      <c r="V3" s="209"/>
-      <c r="W3" s="209"/>
-      <c r="X3" s="209"/>
-      <c r="Y3" s="209"/>
-      <c r="Z3" s="209"/>
+      <c r="Q3" s="208"/>
+      <c r="R3" s="208"/>
+      <c r="S3" s="208"/>
+      <c r="T3" s="208"/>
+      <c r="U3" s="208"/>
+      <c r="V3" s="208"/>
+      <c r="W3" s="208"/>
+      <c r="X3" s="208"/>
+      <c r="Y3" s="208"/>
+      <c r="Z3" s="208"/>
       <c r="AA3" s="146"/>
       <c r="AB3"/>
-      <c r="AC3" s="209" t="s">
+      <c r="AC3" s="208" t="s">
         <v>184</v>
       </c>
-      <c r="AD3" s="209"/>
-      <c r="AE3" s="209"/>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="209"/>
-      <c r="AH3" s="209"/>
-      <c r="AI3" s="209"/>
-      <c r="AJ3" s="209"/>
-      <c r="AK3" s="209"/>
-      <c r="AL3" s="209"/>
-      <c r="AM3" s="209"/>
+      <c r="AD3" s="208"/>
+      <c r="AE3" s="208"/>
+      <c r="AF3" s="208"/>
+      <c r="AG3" s="208"/>
+      <c r="AH3" s="208"/>
+      <c r="AI3" s="208"/>
+      <c r="AJ3" s="208"/>
+      <c r="AK3" s="208"/>
+      <c r="AL3" s="208"/>
+      <c r="AM3" s="208"/>
       <c r="AN3" s="146"/>
       <c r="AO3"/>
     </row>
@@ -21484,19 +21484,19 @@
       <c r="Z4" s="75"/>
       <c r="AA4" s="146"/>
       <c r="AB4"/>
-      <c r="AC4" s="209" t="s">
+      <c r="AC4" s="208" t="s">
         <v>57</v>
       </c>
-      <c r="AD4" s="209"/>
-      <c r="AE4" s="209"/>
-      <c r="AF4" s="209"/>
-      <c r="AG4" s="209"/>
-      <c r="AH4" s="209"/>
-      <c r="AI4" s="209"/>
-      <c r="AJ4" s="209"/>
-      <c r="AK4" s="209"/>
-      <c r="AL4" s="209"/>
-      <c r="AM4" s="209"/>
+      <c r="AD4" s="208"/>
+      <c r="AE4" s="208"/>
+      <c r="AF4" s="208"/>
+      <c r="AG4" s="208"/>
+      <c r="AH4" s="208"/>
+      <c r="AI4" s="208"/>
+      <c r="AJ4" s="208"/>
+      <c r="AK4" s="208"/>
+      <c r="AL4" s="208"/>
+      <c r="AM4" s="208"/>
       <c r="AN4" s="146"/>
       <c r="AO4"/>
     </row>
@@ -21734,14 +21734,14 @@
       <c r="D11" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="210" t="s">
+      <c r="F11" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="210"/>
-      <c r="H11" s="210"/>
-      <c r="I11" s="210"/>
-      <c r="J11" s="210"/>
-      <c r="K11" s="210"/>
+      <c r="G11" s="209"/>
+      <c r="H11" s="209"/>
+      <c r="I11" s="209"/>
+      <c r="J11" s="209"/>
+      <c r="K11" s="209"/>
       <c r="M11" s="53" t="s">
         <v>17</v>
       </c>
@@ -21752,14 +21752,14 @@
       <c r="Q11" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="S11" s="210" t="s">
+      <c r="S11" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="T11" s="210"/>
-      <c r="U11" s="210"/>
-      <c r="V11" s="210"/>
-      <c r="W11" s="210"/>
-      <c r="X11" s="210"/>
+      <c r="T11" s="209"/>
+      <c r="U11" s="209"/>
+      <c r="V11" s="209"/>
+      <c r="W11" s="209"/>
+      <c r="X11" s="209"/>
       <c r="Z11" s="53" t="s">
         <v>17</v>
       </c>
@@ -21771,14 +21771,14 @@
         <v>15</v>
       </c>
       <c r="AE11" s="1"/>
-      <c r="AF11" s="211" t="s">
+      <c r="AF11" s="214" t="s">
         <v>16</v>
       </c>
-      <c r="AG11" s="211"/>
-      <c r="AH11" s="211"/>
-      <c r="AI11" s="211"/>
-      <c r="AJ11" s="211"/>
-      <c r="AK11" s="211"/>
+      <c r="AG11" s="214"/>
+      <c r="AH11" s="214"/>
+      <c r="AI11" s="214"/>
+      <c r="AJ11" s="214"/>
+      <c r="AK11" s="214"/>
       <c r="AL11" s="19"/>
       <c r="AM11" s="4" t="s">
         <v>17</v>
@@ -22123,10 +22123,10 @@
       <c r="Q18" s="36" t="s">
         <v>272</v>
       </c>
-      <c r="S18" s="55"/>
-      <c r="T18" s="155">
+      <c r="S18" s="155">
         <v>7</v>
       </c>
+      <c r="T18" s="55"/>
       <c r="U18" s="56"/>
       <c r="V18" s="56"/>
       <c r="W18" s="56"/>
@@ -22171,7 +22171,7 @@
       </c>
       <c r="Q19" s="36"/>
       <c r="S19" s="56"/>
-      <c r="T19" s="56"/>
+      <c r="T19" s="55"/>
       <c r="U19" s="56"/>
       <c r="V19" s="56"/>
       <c r="W19" s="56"/>
@@ -22218,7 +22218,7 @@
         <v>257</v>
       </c>
       <c r="S20" s="56"/>
-      <c r="T20" s="56"/>
+      <c r="T20" s="55"/>
       <c r="U20" s="56"/>
       <c r="V20" s="56"/>
       <c r="W20" s="60"/>
@@ -22271,7 +22271,7 @@
         <v>256</v>
       </c>
       <c r="S21" s="56"/>
-      <c r="T21" s="56"/>
+      <c r="T21" s="55"/>
       <c r="U21" s="56"/>
       <c r="V21" s="155">
         <v>6</v>
@@ -22318,7 +22318,7 @@
       </c>
       <c r="Q22" s="36"/>
       <c r="S22" s="56"/>
-      <c r="T22" s="56"/>
+      <c r="T22" s="55"/>
       <c r="U22" s="56"/>
       <c r="V22" s="56"/>
       <c r="W22" s="56"/>
@@ -22365,7 +22365,7 @@
         <v>255</v>
       </c>
       <c r="S23" s="56"/>
-      <c r="T23" s="56"/>
+      <c r="T23" s="55"/>
       <c r="U23" s="56"/>
       <c r="V23" s="56"/>
       <c r="W23" s="56"/>
@@ -22418,7 +22418,7 @@
         <v>266</v>
       </c>
       <c r="S24" s="56"/>
-      <c r="T24" s="56"/>
+      <c r="T24" s="55"/>
       <c r="U24" s="56"/>
       <c r="V24" s="56"/>
       <c r="W24" s="155">
@@ -22463,7 +22463,7 @@
       </c>
       <c r="Q25" s="36"/>
       <c r="S25" s="56"/>
-      <c r="T25" s="56"/>
+      <c r="T25" s="55"/>
       <c r="U25" s="56"/>
       <c r="V25" s="56"/>
       <c r="W25" s="56"/>
@@ -22520,8 +22520,8 @@
       <c r="Q26" s="36" t="s">
         <v>274</v>
       </c>
-      <c r="S26" s="55"/>
-      <c r="T26" s="62"/>
+      <c r="S26" s="62"/>
+      <c r="T26" s="55"/>
       <c r="U26" s="55"/>
       <c r="V26" s="55"/>
       <c r="W26" s="55"/>
@@ -22824,86 +22824,86 @@
     </row>
     <row r="36" spans="1:41" ht="19">
       <c r="A36" s="146"/>
-      <c r="D36" s="207" t="s">
+      <c r="D36" s="227" t="s">
         <v>24</v>
       </c>
-      <c r="E36" s="208"/>
-      <c r="F36" s="208"/>
-      <c r="G36" s="208"/>
-      <c r="H36" s="208"/>
-      <c r="I36" s="208"/>
-      <c r="J36" s="208"/>
-      <c r="K36" s="208"/>
-      <c r="L36" s="208"/>
-      <c r="M36" s="208"/>
+      <c r="E36" s="228"/>
+      <c r="F36" s="228"/>
+      <c r="G36" s="228"/>
+      <c r="H36" s="228"/>
+      <c r="I36" s="228"/>
+      <c r="J36" s="228"/>
+      <c r="K36" s="228"/>
+      <c r="L36" s="228"/>
+      <c r="M36" s="228"/>
       <c r="N36" s="146"/>
-      <c r="Q36" s="207" t="s">
+      <c r="Q36" s="227" t="s">
         <v>24</v>
       </c>
-      <c r="R36" s="208"/>
-      <c r="S36" s="208"/>
-      <c r="T36" s="208"/>
-      <c r="U36" s="208"/>
-      <c r="V36" s="208"/>
-      <c r="W36" s="208"/>
-      <c r="X36" s="208"/>
-      <c r="Y36" s="208"/>
-      <c r="Z36" s="208"/>
+      <c r="R36" s="228"/>
+      <c r="S36" s="228"/>
+      <c r="T36" s="228"/>
+      <c r="U36" s="228"/>
+      <c r="V36" s="228"/>
+      <c r="W36" s="228"/>
+      <c r="X36" s="228"/>
+      <c r="Y36" s="228"/>
+      <c r="Z36" s="228"/>
       <c r="AA36" s="146"/>
-      <c r="AD36" s="207" t="s">
+      <c r="AD36" s="227" t="s">
         <v>24</v>
       </c>
-      <c r="AE36" s="208"/>
-      <c r="AF36" s="208"/>
-      <c r="AG36" s="208"/>
-      <c r="AH36" s="208"/>
-      <c r="AI36" s="208"/>
-      <c r="AJ36" s="208"/>
-      <c r="AK36" s="208"/>
-      <c r="AL36" s="208"/>
-      <c r="AM36" s="208"/>
+      <c r="AE36" s="228"/>
+      <c r="AF36" s="228"/>
+      <c r="AG36" s="228"/>
+      <c r="AH36" s="228"/>
+      <c r="AI36" s="228"/>
+      <c r="AJ36" s="228"/>
+      <c r="AK36" s="228"/>
+      <c r="AL36" s="228"/>
+      <c r="AM36" s="228"/>
       <c r="AN36" s="146"/>
     </row>
     <row r="37" spans="1:41">
       <c r="A37" s="146"/>
-      <c r="D37" s="206" t="s">
+      <c r="D37" s="226" t="s">
         <v>176</v>
       </c>
-      <c r="E37" s="206"/>
-      <c r="F37" s="206"/>
-      <c r="G37" s="206"/>
-      <c r="H37" s="206"/>
-      <c r="I37" s="206"/>
-      <c r="J37" s="206"/>
-      <c r="K37" s="206"/>
-      <c r="L37" s="206"/>
-      <c r="M37" s="206"/>
+      <c r="E37" s="226"/>
+      <c r="F37" s="226"/>
+      <c r="G37" s="226"/>
+      <c r="H37" s="226"/>
+      <c r="I37" s="226"/>
+      <c r="J37" s="226"/>
+      <c r="K37" s="226"/>
+      <c r="L37" s="226"/>
+      <c r="M37" s="226"/>
       <c r="N37" s="146"/>
-      <c r="Q37" s="206" t="s">
+      <c r="Q37" s="226" t="s">
         <v>176</v>
       </c>
-      <c r="R37" s="206"/>
-      <c r="S37" s="206"/>
-      <c r="T37" s="206"/>
-      <c r="U37" s="206"/>
-      <c r="V37" s="206"/>
-      <c r="W37" s="206"/>
-      <c r="X37" s="206"/>
-      <c r="Y37" s="206"/>
-      <c r="Z37" s="206"/>
+      <c r="R37" s="226"/>
+      <c r="S37" s="226"/>
+      <c r="T37" s="226"/>
+      <c r="U37" s="226"/>
+      <c r="V37" s="226"/>
+      <c r="W37" s="226"/>
+      <c r="X37" s="226"/>
+      <c r="Y37" s="226"/>
+      <c r="Z37" s="226"/>
       <c r="AA37" s="146"/>
-      <c r="AD37" s="206" t="s">
+      <c r="AD37" s="226" t="s">
         <v>176</v>
       </c>
-      <c r="AE37" s="206"/>
-      <c r="AF37" s="206"/>
-      <c r="AG37" s="206"/>
-      <c r="AH37" s="206"/>
-      <c r="AI37" s="206"/>
-      <c r="AJ37" s="206"/>
-      <c r="AK37" s="206"/>
-      <c r="AL37" s="206"/>
-      <c r="AM37" s="206"/>
+      <c r="AE37" s="226"/>
+      <c r="AF37" s="226"/>
+      <c r="AG37" s="226"/>
+      <c r="AH37" s="226"/>
+      <c r="AI37" s="226"/>
+      <c r="AJ37" s="226"/>
+      <c r="AK37" s="226"/>
+      <c r="AL37" s="226"/>
+      <c r="AM37" s="226"/>
       <c r="AN37" s="146"/>
     </row>
     <row r="38" spans="1:41">
@@ -23966,6 +23966,12 @@
     <row r="81" ht="17" thickTop="1"/>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="AD37:AM37"/>
+    <mergeCell ref="D36:M36"/>
+    <mergeCell ref="D37:M37"/>
+    <mergeCell ref="Q36:Z36"/>
+    <mergeCell ref="Q37:Z37"/>
+    <mergeCell ref="AD36:AM36"/>
     <mergeCell ref="C3:M3"/>
     <mergeCell ref="P3:Z3"/>
     <mergeCell ref="AC3:AM3"/>
@@ -23973,12 +23979,6 @@
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="S11:X11"/>
     <mergeCell ref="AF11:AK11"/>
-    <mergeCell ref="AD37:AM37"/>
-    <mergeCell ref="D36:M36"/>
-    <mergeCell ref="D37:M37"/>
-    <mergeCell ref="Q36:Z36"/>
-    <mergeCell ref="Q37:Z37"/>
-    <mergeCell ref="AD36:AM36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D37" r:id="rId1" xr:uid="{E918FEAF-0D24-E348-B153-6B5AA2FA18F9}"/>
@@ -24075,46 +24075,46 @@
     <row r="3" spans="1:38" s="74" customFormat="1" ht="19">
       <c r="A3" s="146"/>
       <c r="B3"/>
-      <c r="C3" s="209" t="s">
+      <c r="C3" s="208" t="s">
         <v>359</v>
       </c>
-      <c r="D3" s="209"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="209"/>
-      <c r="G3" s="209"/>
-      <c r="H3" s="209"/>
-      <c r="I3" s="209"/>
-      <c r="J3" s="209"/>
-      <c r="K3" s="209"/>
-      <c r="L3" s="209"/>
+      <c r="D3" s="208"/>
+      <c r="E3" s="208"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="208"/>
+      <c r="H3" s="208"/>
+      <c r="I3" s="208"/>
+      <c r="J3" s="208"/>
+      <c r="K3" s="208"/>
+      <c r="L3" s="208"/>
       <c r="M3" s="146"/>
       <c r="N3"/>
-      <c r="O3" s="209" t="s">
+      <c r="O3" s="208" t="s">
         <v>358</v>
       </c>
-      <c r="P3" s="209"/>
-      <c r="Q3" s="209"/>
-      <c r="R3" s="209"/>
-      <c r="S3" s="209"/>
-      <c r="T3" s="209"/>
-      <c r="U3" s="209"/>
-      <c r="V3" s="209"/>
-      <c r="W3" s="209"/>
-      <c r="X3" s="209"/>
+      <c r="P3" s="208"/>
+      <c r="Q3" s="208"/>
+      <c r="R3" s="208"/>
+      <c r="S3" s="208"/>
+      <c r="T3" s="208"/>
+      <c r="U3" s="208"/>
+      <c r="V3" s="208"/>
+      <c r="W3" s="208"/>
+      <c r="X3" s="208"/>
       <c r="Y3" s="146"/>
       <c r="Z3"/>
-      <c r="AA3" s="209" t="s">
+      <c r="AA3" s="208" t="s">
         <v>360</v>
       </c>
-      <c r="AB3" s="209"/>
-      <c r="AC3" s="209"/>
-      <c r="AD3" s="209"/>
-      <c r="AE3" s="209"/>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="209"/>
-      <c r="AH3" s="209"/>
-      <c r="AI3" s="209"/>
-      <c r="AJ3" s="209"/>
+      <c r="AB3" s="208"/>
+      <c r="AC3" s="208"/>
+      <c r="AD3" s="208"/>
+      <c r="AE3" s="208"/>
+      <c r="AF3" s="208"/>
+      <c r="AG3" s="208"/>
+      <c r="AH3" s="208"/>
+      <c r="AI3" s="208"/>
+      <c r="AJ3" s="208"/>
       <c r="AK3" s="146"/>
       <c r="AL3"/>
     </row>
@@ -24346,13 +24346,13 @@
       <c r="D10" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="210" t="s">
+      <c r="F10" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="210"/>
-      <c r="H10" s="210"/>
-      <c r="I10" s="210"/>
-      <c r="J10" s="210"/>
+      <c r="G10" s="209"/>
+      <c r="H10" s="209"/>
+      <c r="I10" s="209"/>
+      <c r="J10" s="209"/>
       <c r="L10" s="53" t="s">
         <v>17</v>
       </c>
@@ -24363,13 +24363,13 @@
       <c r="P10" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="R10" s="210" t="s">
+      <c r="R10" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="S10" s="210"/>
-      <c r="T10" s="210"/>
-      <c r="U10" s="210"/>
-      <c r="V10" s="210"/>
+      <c r="S10" s="209"/>
+      <c r="T10" s="209"/>
+      <c r="U10" s="209"/>
+      <c r="V10" s="209"/>
       <c r="X10" s="53" t="s">
         <v>17</v>
       </c>
@@ -24380,11 +24380,11 @@
       <c r="AB10" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="AD10" s="210"/>
-      <c r="AE10" s="210"/>
-      <c r="AF10" s="210"/>
-      <c r="AG10" s="210"/>
-      <c r="AH10" s="210"/>
+      <c r="AD10" s="209"/>
+      <c r="AE10" s="209"/>
+      <c r="AF10" s="209"/>
+      <c r="AG10" s="209"/>
+      <c r="AH10" s="209"/>
       <c r="AJ10" s="53" t="s">
         <v>17</v>
       </c>
@@ -25007,84 +25007,84 @@
     <row r="25" spans="1:38" s="1" customFormat="1">
       <c r="A25" s="146"/>
       <c r="C25" s="201"/>
-      <c r="D25" s="221" t="s">
+      <c r="D25" s="206" t="s">
         <v>24</v>
       </c>
-      <c r="E25" s="221"/>
-      <c r="F25" s="221"/>
-      <c r="G25" s="221"/>
-      <c r="H25" s="221"/>
-      <c r="I25" s="221"/>
-      <c r="J25" s="221"/>
-      <c r="K25" s="221"/>
-      <c r="L25" s="221"/>
+      <c r="E25" s="206"/>
+      <c r="F25" s="206"/>
+      <c r="G25" s="206"/>
+      <c r="H25" s="206"/>
+      <c r="I25" s="206"/>
+      <c r="J25" s="206"/>
+      <c r="K25" s="206"/>
+      <c r="L25" s="206"/>
       <c r="M25" s="146"/>
-      <c r="P25" s="221" t="s">
+      <c r="P25" s="206" t="s">
         <v>24</v>
       </c>
-      <c r="Q25" s="221"/>
-      <c r="R25" s="221"/>
-      <c r="S25" s="221"/>
-      <c r="T25" s="221"/>
-      <c r="U25" s="221"/>
-      <c r="V25" s="221"/>
-      <c r="W25" s="221"/>
-      <c r="X25" s="221"/>
+      <c r="Q25" s="206"/>
+      <c r="R25" s="206"/>
+      <c r="S25" s="206"/>
+      <c r="T25" s="206"/>
+      <c r="U25" s="206"/>
+      <c r="V25" s="206"/>
+      <c r="W25" s="206"/>
+      <c r="X25" s="206"/>
       <c r="Y25" s="146"/>
-      <c r="AB25" s="221" t="s">
+      <c r="AB25" s="206" t="s">
         <v>24</v>
       </c>
-      <c r="AC25" s="221"/>
-      <c r="AD25" s="221"/>
-      <c r="AE25" s="221"/>
-      <c r="AF25" s="221"/>
-      <c r="AG25" s="221"/>
-      <c r="AH25" s="221"/>
-      <c r="AI25" s="221"/>
-      <c r="AJ25" s="221"/>
+      <c r="AC25" s="206"/>
+      <c r="AD25" s="206"/>
+      <c r="AE25" s="206"/>
+      <c r="AF25" s="206"/>
+      <c r="AG25" s="206"/>
+      <c r="AH25" s="206"/>
+      <c r="AI25" s="206"/>
+      <c r="AJ25" s="206"/>
       <c r="AK25" s="146"/>
     </row>
     <row r="26" spans="1:38" s="1" customFormat="1">
       <c r="A26" s="146"/>
       <c r="B26" s="19"/>
       <c r="C26" s="201"/>
-      <c r="D26" s="228" t="s">
+      <c r="D26" s="207" t="s">
         <v>176</v>
       </c>
-      <c r="E26" s="228"/>
-      <c r="F26" s="228"/>
-      <c r="G26" s="228"/>
-      <c r="H26" s="228"/>
-      <c r="I26" s="228"/>
-      <c r="J26" s="228"/>
-      <c r="K26" s="228"/>
-      <c r="L26" s="228"/>
+      <c r="E26" s="207"/>
+      <c r="F26" s="207"/>
+      <c r="G26" s="207"/>
+      <c r="H26" s="207"/>
+      <c r="I26" s="207"/>
+      <c r="J26" s="207"/>
+      <c r="K26" s="207"/>
+      <c r="L26" s="207"/>
       <c r="M26" s="146"/>
       <c r="N26" s="19"/>
-      <c r="P26" s="228" t="s">
+      <c r="P26" s="207" t="s">
         <v>176</v>
       </c>
-      <c r="Q26" s="228"/>
-      <c r="R26" s="228"/>
-      <c r="S26" s="228"/>
-      <c r="T26" s="228"/>
-      <c r="U26" s="228"/>
-      <c r="V26" s="228"/>
-      <c r="W26" s="228"/>
-      <c r="X26" s="228"/>
+      <c r="Q26" s="207"/>
+      <c r="R26" s="207"/>
+      <c r="S26" s="207"/>
+      <c r="T26" s="207"/>
+      <c r="U26" s="207"/>
+      <c r="V26" s="207"/>
+      <c r="W26" s="207"/>
+      <c r="X26" s="207"/>
       <c r="Y26" s="146"/>
       <c r="Z26" s="19"/>
-      <c r="AB26" s="228" t="s">
+      <c r="AB26" s="207" t="s">
         <v>176</v>
       </c>
-      <c r="AC26" s="228"/>
-      <c r="AD26" s="228"/>
-      <c r="AE26" s="228"/>
-      <c r="AF26" s="228"/>
-      <c r="AG26" s="228"/>
-      <c r="AH26" s="228"/>
-      <c r="AI26" s="228"/>
-      <c r="AJ26" s="228"/>
+      <c r="AC26" s="207"/>
+      <c r="AD26" s="207"/>
+      <c r="AE26" s="207"/>
+      <c r="AF26" s="207"/>
+      <c r="AG26" s="207"/>
+      <c r="AH26" s="207"/>
+      <c r="AI26" s="207"/>
+      <c r="AJ26" s="207"/>
       <c r="AK26" s="146"/>
       <c r="AL26" s="19"/>
     </row>
@@ -25938,18 +25938,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="C3:L3"/>
+    <mergeCell ref="O3:X3"/>
+    <mergeCell ref="AA3:AJ3"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="AD10:AH10"/>
     <mergeCell ref="D25:L25"/>
     <mergeCell ref="P25:X25"/>
     <mergeCell ref="AB25:AJ25"/>
     <mergeCell ref="D26:L26"/>
     <mergeCell ref="P26:X26"/>
     <mergeCell ref="AB26:AJ26"/>
-    <mergeCell ref="C3:L3"/>
-    <mergeCell ref="O3:X3"/>
-    <mergeCell ref="AA3:AJ3"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="AD10:AH10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D26" r:id="rId1" xr:uid="{C04FEEE9-A64B-DC4D-B76B-186D1E9AA236}"/>
@@ -26061,61 +26061,61 @@
     <row r="3" spans="1:53" s="74" customFormat="1" ht="19">
       <c r="A3" s="146"/>
       <c r="B3"/>
-      <c r="C3" s="209" t="s">
+      <c r="C3" s="208" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="209"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="209"/>
-      <c r="G3" s="209"/>
-      <c r="H3" s="209"/>
-      <c r="I3" s="209"/>
-      <c r="J3" s="209"/>
-      <c r="K3" s="209"/>
-      <c r="L3" s="209"/>
-      <c r="M3" s="209"/>
-      <c r="N3" s="209"/>
-      <c r="O3" s="209"/>
-      <c r="P3" s="209"/>
-      <c r="Q3" s="209"/>
+      <c r="D3" s="208"/>
+      <c r="E3" s="208"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="208"/>
+      <c r="H3" s="208"/>
+      <c r="I3" s="208"/>
+      <c r="J3" s="208"/>
+      <c r="K3" s="208"/>
+      <c r="L3" s="208"/>
+      <c r="M3" s="208"/>
+      <c r="N3" s="208"/>
+      <c r="O3" s="208"/>
+      <c r="P3" s="208"/>
+      <c r="Q3" s="208"/>
       <c r="R3" s="146"/>
       <c r="S3"/>
-      <c r="T3" s="209" t="s">
+      <c r="T3" s="208" t="s">
         <v>61</v>
       </c>
-      <c r="U3" s="209"/>
-      <c r="V3" s="209"/>
-      <c r="W3" s="209"/>
-      <c r="X3" s="209"/>
-      <c r="Y3" s="209"/>
-      <c r="Z3" s="209"/>
-      <c r="AA3" s="209"/>
-      <c r="AB3" s="209"/>
-      <c r="AC3" s="209"/>
-      <c r="AD3" s="209"/>
-      <c r="AE3" s="209"/>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="209"/>
-      <c r="AH3" s="209"/>
+      <c r="U3" s="208"/>
+      <c r="V3" s="208"/>
+      <c r="W3" s="208"/>
+      <c r="X3" s="208"/>
+      <c r="Y3" s="208"/>
+      <c r="Z3" s="208"/>
+      <c r="AA3" s="208"/>
+      <c r="AB3" s="208"/>
+      <c r="AC3" s="208"/>
+      <c r="AD3" s="208"/>
+      <c r="AE3" s="208"/>
+      <c r="AF3" s="208"/>
+      <c r="AG3" s="208"/>
+      <c r="AH3" s="208"/>
       <c r="AI3" s="146"/>
       <c r="AJ3"/>
-      <c r="AK3" s="209" t="s">
+      <c r="AK3" s="208" t="s">
         <v>62</v>
       </c>
-      <c r="AL3" s="209"/>
-      <c r="AM3" s="209"/>
-      <c r="AN3" s="209"/>
-      <c r="AO3" s="209"/>
-      <c r="AP3" s="209"/>
-      <c r="AQ3" s="209"/>
-      <c r="AR3" s="209"/>
-      <c r="AS3" s="209"/>
-      <c r="AT3" s="209"/>
-      <c r="AU3" s="209"/>
-      <c r="AV3" s="209"/>
-      <c r="AW3" s="209"/>
-      <c r="AX3" s="209"/>
-      <c r="AY3" s="209"/>
+      <c r="AL3" s="208"/>
+      <c r="AM3" s="208"/>
+      <c r="AN3" s="208"/>
+      <c r="AO3" s="208"/>
+      <c r="AP3" s="208"/>
+      <c r="AQ3" s="208"/>
+      <c r="AR3" s="208"/>
+      <c r="AS3" s="208"/>
+      <c r="AT3" s="208"/>
+      <c r="AU3" s="208"/>
+      <c r="AV3" s="208"/>
+      <c r="AW3" s="208"/>
+      <c r="AX3" s="208"/>
+      <c r="AY3" s="208"/>
       <c r="AZ3" s="146"/>
       <c r="BA3"/>
     </row>
@@ -26464,18 +26464,18 @@
       <c r="D10" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="210" t="s">
+      <c r="F10" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="210"/>
-      <c r="H10" s="210"/>
-      <c r="I10" s="210"/>
-      <c r="J10" s="210"/>
-      <c r="K10" s="210"/>
-      <c r="L10" s="210"/>
-      <c r="M10" s="210"/>
-      <c r="N10" s="210"/>
-      <c r="O10" s="210"/>
+      <c r="G10" s="209"/>
+      <c r="H10" s="209"/>
+      <c r="I10" s="209"/>
+      <c r="J10" s="209"/>
+      <c r="K10" s="209"/>
+      <c r="L10" s="209"/>
+      <c r="M10" s="209"/>
+      <c r="N10" s="209"/>
+      <c r="O10" s="209"/>
       <c r="Q10" s="53" t="s">
         <v>17</v>
       </c>
@@ -26486,18 +26486,18 @@
       <c r="U10" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="W10" s="210" t="s">
+      <c r="W10" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="X10" s="210"/>
-      <c r="Y10" s="210"/>
-      <c r="Z10" s="210"/>
-      <c r="AA10" s="210"/>
-      <c r="AB10" s="210"/>
-      <c r="AC10" s="210"/>
-      <c r="AD10" s="210"/>
-      <c r="AE10" s="210"/>
-      <c r="AF10" s="210"/>
+      <c r="X10" s="209"/>
+      <c r="Y10" s="209"/>
+      <c r="Z10" s="209"/>
+      <c r="AA10" s="209"/>
+      <c r="AB10" s="209"/>
+      <c r="AC10" s="209"/>
+      <c r="AD10" s="209"/>
+      <c r="AE10" s="209"/>
+      <c r="AF10" s="209"/>
       <c r="AH10" s="53" t="s">
         <v>17</v>
       </c>
@@ -26508,18 +26508,18 @@
       <c r="AL10" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="AN10" s="210" t="s">
+      <c r="AN10" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="AO10" s="210"/>
-      <c r="AP10" s="210"/>
-      <c r="AQ10" s="210"/>
-      <c r="AR10" s="210"/>
-      <c r="AS10" s="210"/>
-      <c r="AT10" s="210"/>
-      <c r="AU10" s="210"/>
-      <c r="AV10" s="210"/>
-      <c r="AW10" s="210"/>
+      <c r="AO10" s="209"/>
+      <c r="AP10" s="209"/>
+      <c r="AQ10" s="209"/>
+      <c r="AR10" s="209"/>
+      <c r="AS10" s="209"/>
+      <c r="AT10" s="209"/>
+      <c r="AU10" s="209"/>
+      <c r="AV10" s="209"/>
+      <c r="AW10" s="209"/>
       <c r="AY10" s="53" t="s">
         <v>17</v>
       </c>
@@ -28117,111 +28117,111 @@
     <row r="35" spans="1:53" s="1" customFormat="1">
       <c r="A35" s="146"/>
       <c r="C35" s="202"/>
-      <c r="D35" s="221" t="s">
+      <c r="D35" s="206" t="s">
         <v>239</v>
       </c>
-      <c r="E35" s="221"/>
-      <c r="F35" s="221"/>
-      <c r="G35" s="221"/>
-      <c r="H35" s="221"/>
-      <c r="I35" s="221"/>
-      <c r="J35" s="221"/>
-      <c r="K35" s="221"/>
-      <c r="L35" s="221"/>
-      <c r="M35" s="221"/>
-      <c r="N35" s="221"/>
-      <c r="O35" s="221"/>
-      <c r="P35" s="221"/>
-      <c r="Q35" s="221"/>
+      <c r="E35" s="206"/>
+      <c r="F35" s="206"/>
+      <c r="G35" s="206"/>
+      <c r="H35" s="206"/>
+      <c r="I35" s="206"/>
+      <c r="J35" s="206"/>
+      <c r="K35" s="206"/>
+      <c r="L35" s="206"/>
+      <c r="M35" s="206"/>
+      <c r="N35" s="206"/>
+      <c r="O35" s="206"/>
+      <c r="P35" s="206"/>
+      <c r="Q35" s="206"/>
       <c r="R35" s="146"/>
-      <c r="U35" s="221" t="s">
+      <c r="U35" s="206" t="s">
         <v>239</v>
       </c>
-      <c r="V35" s="221"/>
-      <c r="W35" s="221"/>
-      <c r="X35" s="221"/>
-      <c r="Y35" s="221"/>
-      <c r="Z35" s="221"/>
-      <c r="AA35" s="221"/>
-      <c r="AB35" s="221"/>
-      <c r="AC35" s="221"/>
-      <c r="AD35" s="221"/>
-      <c r="AE35" s="221"/>
-      <c r="AF35" s="221"/>
-      <c r="AG35" s="221"/>
-      <c r="AH35" s="221"/>
+      <c r="V35" s="206"/>
+      <c r="W35" s="206"/>
+      <c r="X35" s="206"/>
+      <c r="Y35" s="206"/>
+      <c r="Z35" s="206"/>
+      <c r="AA35" s="206"/>
+      <c r="AB35" s="206"/>
+      <c r="AC35" s="206"/>
+      <c r="AD35" s="206"/>
+      <c r="AE35" s="206"/>
+      <c r="AF35" s="206"/>
+      <c r="AG35" s="206"/>
+      <c r="AH35" s="206"/>
       <c r="AI35" s="146"/>
-      <c r="AL35" s="221" t="s">
+      <c r="AL35" s="206" t="s">
         <v>239</v>
       </c>
-      <c r="AM35" s="221"/>
-      <c r="AN35" s="221"/>
-      <c r="AO35" s="221"/>
-      <c r="AP35" s="221"/>
-      <c r="AQ35" s="221"/>
-      <c r="AR35" s="221"/>
-      <c r="AS35" s="221"/>
-      <c r="AT35" s="221"/>
-      <c r="AU35" s="221"/>
-      <c r="AV35" s="221"/>
-      <c r="AW35" s="221"/>
-      <c r="AX35" s="221"/>
-      <c r="AY35" s="221"/>
+      <c r="AM35" s="206"/>
+      <c r="AN35" s="206"/>
+      <c r="AO35" s="206"/>
+      <c r="AP35" s="206"/>
+      <c r="AQ35" s="206"/>
+      <c r="AR35" s="206"/>
+      <c r="AS35" s="206"/>
+      <c r="AT35" s="206"/>
+      <c r="AU35" s="206"/>
+      <c r="AV35" s="206"/>
+      <c r="AW35" s="206"/>
+      <c r="AX35" s="206"/>
+      <c r="AY35" s="206"/>
       <c r="AZ35" s="146"/>
     </row>
     <row r="36" spans="1:53" s="1" customFormat="1">
       <c r="A36" s="146"/>
       <c r="C36" s="202"/>
-      <c r="D36" s="228" t="s">
+      <c r="D36" s="207" t="s">
         <v>176</v>
       </c>
-      <c r="E36" s="228"/>
-      <c r="F36" s="228"/>
-      <c r="G36" s="228"/>
-      <c r="H36" s="228"/>
-      <c r="I36" s="228"/>
-      <c r="J36" s="228"/>
-      <c r="K36" s="228"/>
-      <c r="L36" s="228"/>
-      <c r="M36" s="228"/>
-      <c r="N36" s="228"/>
-      <c r="O36" s="228"/>
-      <c r="P36" s="228"/>
-      <c r="Q36" s="228"/>
+      <c r="E36" s="207"/>
+      <c r="F36" s="207"/>
+      <c r="G36" s="207"/>
+      <c r="H36" s="207"/>
+      <c r="I36" s="207"/>
+      <c r="J36" s="207"/>
+      <c r="K36" s="207"/>
+      <c r="L36" s="207"/>
+      <c r="M36" s="207"/>
+      <c r="N36" s="207"/>
+      <c r="O36" s="207"/>
+      <c r="P36" s="207"/>
+      <c r="Q36" s="207"/>
       <c r="R36" s="146"/>
-      <c r="U36" s="228" t="s">
+      <c r="U36" s="207" t="s">
         <v>176</v>
       </c>
-      <c r="V36" s="228"/>
-      <c r="W36" s="228"/>
-      <c r="X36" s="228"/>
-      <c r="Y36" s="228"/>
-      <c r="Z36" s="228"/>
-      <c r="AA36" s="228"/>
-      <c r="AB36" s="228"/>
-      <c r="AC36" s="228"/>
-      <c r="AD36" s="228"/>
-      <c r="AE36" s="228"/>
-      <c r="AF36" s="228"/>
-      <c r="AG36" s="228"/>
-      <c r="AH36" s="228"/>
+      <c r="V36" s="207"/>
+      <c r="W36" s="207"/>
+      <c r="X36" s="207"/>
+      <c r="Y36" s="207"/>
+      <c r="Z36" s="207"/>
+      <c r="AA36" s="207"/>
+      <c r="AB36" s="207"/>
+      <c r="AC36" s="207"/>
+      <c r="AD36" s="207"/>
+      <c r="AE36" s="207"/>
+      <c r="AF36" s="207"/>
+      <c r="AG36" s="207"/>
+      <c r="AH36" s="207"/>
       <c r="AI36" s="146"/>
-      <c r="AL36" s="228" t="s">
+      <c r="AL36" s="207" t="s">
         <v>176</v>
       </c>
-      <c r="AM36" s="228"/>
-      <c r="AN36" s="228"/>
-      <c r="AO36" s="228"/>
-      <c r="AP36" s="228"/>
-      <c r="AQ36" s="228"/>
-      <c r="AR36" s="228"/>
-      <c r="AS36" s="228"/>
-      <c r="AT36" s="228"/>
-      <c r="AU36" s="228"/>
-      <c r="AV36" s="228"/>
-      <c r="AW36" s="228"/>
-      <c r="AX36" s="228"/>
-      <c r="AY36" s="228"/>
+      <c r="AM36" s="207"/>
+      <c r="AN36" s="207"/>
+      <c r="AO36" s="207"/>
+      <c r="AP36" s="207"/>
+      <c r="AQ36" s="207"/>
+      <c r="AR36" s="207"/>
+      <c r="AS36" s="207"/>
+      <c r="AT36" s="207"/>
+      <c r="AU36" s="207"/>
+      <c r="AV36" s="207"/>
+      <c r="AW36" s="207"/>
+      <c r="AX36" s="207"/>
+      <c r="AY36" s="207"/>
       <c r="AZ36" s="146"/>
     </row>
     <row r="37" spans="1:53" s="1" customFormat="1">
@@ -30239,18 +30239,18 @@
     <row r="90" spans="1:52" ht="17" thickTop="1"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="D35:Q35"/>
+    <mergeCell ref="D36:Q36"/>
+    <mergeCell ref="U35:AH35"/>
+    <mergeCell ref="U36:AH36"/>
+    <mergeCell ref="AL35:AY35"/>
+    <mergeCell ref="AL36:AY36"/>
     <mergeCell ref="C3:Q3"/>
     <mergeCell ref="T3:AH3"/>
     <mergeCell ref="AK3:AY3"/>
     <mergeCell ref="F10:O10"/>
     <mergeCell ref="W10:AF10"/>
     <mergeCell ref="AN10:AW10"/>
-    <mergeCell ref="D35:Q35"/>
-    <mergeCell ref="D36:Q36"/>
-    <mergeCell ref="U35:AH35"/>
-    <mergeCell ref="U36:AH36"/>
-    <mergeCell ref="AL35:AY35"/>
-    <mergeCell ref="AL36:AY36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D36" r:id="rId1" xr:uid="{829AD50E-953F-7542-AA9E-869853F367F6}"/>

</xml_diff>